<commit_message>
Dial sample assumptions to a realistic SaaS base case
Revenue growth 35% -> 16% (fade 3%/yr), EBITDA margin 27% -> 26%,
net margin 14% -> 13.5%, peer multiples trimmed. Consensus revenue/EBITDA/NI
aligned to a ~15% grower. Result: DCF fair value $45.86 vs $45 price (+1.9%),
blended surprise +2.5% (slight beat) — defensible base case. Re-exported xlsx.
</commit_message>
<xml_diff>
--- a/Sector_Consensus_vs_My_Model.xlsx
+++ b/Sector_Consensus_vs_My_Model.xlsx
@@ -649,13 +649,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="7">
-    <numFmt numFmtId="164" formatCode="$#,##0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.0&quot;x&quot;"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
-    <numFmt numFmtId="168" formatCode="MMM D, YYYY"/>
-    <numFmt numFmtId="169" formatCode="#,##0.0"/>
-    <numFmt numFmtId="170" formatCode="#,##0"/>
+    <numFmt numFmtId="167" formatCode="$#,##0.0"/>
+    <numFmt numFmtId="168" formatCode="#,##0.0"/>
+    <numFmt numFmtId="169" formatCode="#,##0"/>
+    <numFmt numFmtId="170" formatCode="MMM D, YYYY"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -667,22 +667,23 @@
     </font>
     <font>
       <b/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF006100"/>
+    </font>
+    <font>
+      <b/>
       <sz val="14"/>
       <color rgb="FFFFFFFF"/>
     </font>
     <font>
       <b/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-    </font>
-    <font>
-      <color rgb="FF1A1A1A"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
     </font>
     <font>
@@ -692,6 +693,9 @@
     <font>
       <b/>
       <color rgb="FF2E5C9A"/>
+    </font>
+    <font>
+      <color rgb="FF1A1A1A"/>
     </font>
     <font>
       <b/>
@@ -704,10 +708,6 @@
     </font>
     <font>
       <b val="0"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF006100"/>
     </font>
     <font>
       <b/>
@@ -727,8 +727,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F3864"/>
-        <bgColor rgb="FF1F3864"/>
+        <fgColor rgb="FFD9E1F2"/>
+        <bgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -739,26 +739,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F3864"/>
+        <bgColor rgb="FF1F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFF2F6FC"/>
         <bgColor rgb="FFF2F6FC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9E1F2"/>
-        <bgColor rgb="FFD9E1F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF2E5C9A"/>
         <bgColor rgb="FF2E5C9A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -791,83 +791,83 @@
   <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="167" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="167" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="169" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="170" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="170" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="11" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1315,400 +1315,400 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="20" t="s">
         <v>1</v>
       </c>
       <c r="B3" t="str">
         <f>Inputs!D4</f>
         <v>Nimbus Cloud Inc</v>
       </c>
-      <c r="E3" s="17" t="s">
+      <c r="E3" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="45" t="s">
+      <c r="G3" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="17" t="s">
+      <c r="I3" s="20" t="s">
         <v>4</v>
       </c>
       <c r="J3">
         <f>Price</f>
         <v>45</v>
       </c>
-      <c r="K3" s="36"/>
+      <c r="K3" s="44"/>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="20" t="s">
         <v>5</v>
       </c>
       <c r="B4" t="str">
         <f>Inputs!D5</f>
         <v>NIMB</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="E4" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="32">
+      <c r="F4" s="42">
         <f>Inputs!D10</f>
         <v>46231</v>
       </c>
-      <c r="G4" s="32"/>
-      <c r="I4" s="17" t="s">
+      <c r="G4" s="42"/>
+      <c r="I4" s="20" t="s">
         <v>7</v>
       </c>
       <c r="J4">
         <f>Shares</f>
         <v>100</v>
       </c>
-      <c r="K4" s="29"/>
+      <c r="K4" s="35"/>
     </row>
     <row r="6">
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="F6" s="18" t="s">
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="F6" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="J6" s="18" t="s">
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="J6" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
     </row>
     <row r="7">
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="21">
         <f>RevMy</f>
-        <v>1350</v>
-      </c>
-      <c r="D7" s="8"/>
-      <c r="F7" s="19" t="s">
+        <v>1160</v>
+      </c>
+      <c r="D7" s="25"/>
+      <c r="F7" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="16">
+      <c r="G7" s="21">
         <f>EbitdaMy</f>
-        <v>364.5</v>
-      </c>
-      <c r="H7" s="8"/>
-      <c r="J7" s="19" t="s">
+        <v>301.6</v>
+      </c>
+      <c r="H7" s="25"/>
+      <c r="J7" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="K7" s="16">
+      <c r="K7" s="21">
         <f>NiMy</f>
-        <v>189.00000000000003</v>
-      </c>
-      <c r="L7" s="8"/>
+        <v>156.60000000000002</v>
+      </c>
+      <c r="L7" s="25"/>
     </row>
     <row r="8">
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="21">
         <f>ConsRev</f>
-        <v>1300</v>
-      </c>
-      <c r="D8" s="8"/>
-      <c r="F8" s="19" t="s">
+        <v>1150</v>
+      </c>
+      <c r="D8" s="25"/>
+      <c r="F8" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="16">
+      <c r="G8" s="21">
         <f>ConsEBITDA</f>
-        <v>340</v>
-      </c>
-      <c r="H8" s="8"/>
-      <c r="J8" s="19" t="s">
+        <v>295</v>
+      </c>
+      <c r="H8" s="25"/>
+      <c r="J8" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="K8" s="16">
+      <c r="K8" s="21">
         <f>ConsNI</f>
-        <v>175</v>
-      </c>
-      <c r="L8" s="8"/>
+        <v>150</v>
+      </c>
+      <c r="L8" s="25"/>
     </row>
     <row r="9">
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="28">
+      <c r="C9" s="34">
         <f>RevMy/PriorRev-1</f>
-        <v>0.3500000000000001</v>
-      </c>
-      <c r="D9" s="8"/>
-      <c r="F9" s="19" t="s">
+        <v>0.15999999999999992</v>
+      </c>
+      <c r="D9" s="25"/>
+      <c r="F9" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="28">
+      <c r="G9" s="34">
         <f>EbitdaMy/PriorEBITDA-1</f>
-        <v>0.45799999999999996</v>
-      </c>
-      <c r="H9" s="8"/>
-      <c r="J9" s="19" t="s">
+        <v>0.20640000000000014</v>
+      </c>
+      <c r="H9" s="25"/>
+      <c r="J9" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="K9" s="28">
+      <c r="K9" s="34">
         <f>NiMy/PriorNI-1</f>
-        <v>0.5750000000000002</v>
-      </c>
-      <c r="L9" s="8"/>
+        <v>0.30500000000000016</v>
+      </c>
+      <c r="L9" s="25"/>
     </row>
     <row r="10">
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="28">
+      <c r="C10" s="34">
         <f>RevMy/ConsRev-1</f>
-        <v>0.03846153846153855</v>
-      </c>
-      <c r="D10" s="8"/>
-      <c r="F10" s="19" t="s">
+        <v>0.008695652173912993</v>
+      </c>
+      <c r="D10" s="25"/>
+      <c r="F10" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="28">
+      <c r="G10" s="34">
         <f>EbitdaMy/ConsEBITDA-1</f>
-        <v>0.07205882352941173</v>
-      </c>
-      <c r="H10" s="8"/>
-      <c r="J10" s="19" t="s">
+        <v>0.022372881355932295</v>
+      </c>
+      <c r="H10" s="25"/>
+      <c r="J10" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="K10" s="28">
+      <c r="K10" s="34">
         <f>NiMy/ConsNI-1</f>
-        <v>0.08000000000000007</v>
-      </c>
-      <c r="L10" s="8"/>
+        <v>0.04400000000000026</v>
+      </c>
+      <c r="L10" s="25"/>
     </row>
     <row r="11">
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="35" t="str">
+      <c r="C11" s="43" t="str">
         <f>IF(RevMy/ConsRev-1&gt;=BeatThresh,"BEAT",IF(RevMy/ConsRev-1&lt;=MissThresh,"MISS","IN-LINE"))</f>
-        <v>BEAT</v>
-      </c>
-      <c r="D11" s="8"/>
-      <c r="F11" s="19" t="s">
+        <v>IN-LINE</v>
+      </c>
+      <c r="D11" s="25"/>
+      <c r="F11" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="G11" s="35" t="str">
+      <c r="G11" s="43" t="str">
         <f>IF(EbitdaMy/ConsEBITDA-1&gt;=BeatThresh,"BEAT",IF(EbitdaMy/ConsEBITDA-1&lt;=MissThresh,"MISS","IN-LINE"))</f>
         <v>BEAT</v>
       </c>
-      <c r="H11" s="8"/>
-      <c r="J11" s="19" t="s">
+      <c r="H11" s="25"/>
+      <c r="J11" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="K11" s="35" t="str">
+      <c r="K11" s="43" t="str">
         <f>IF(NiMy/ConsNI-1&gt;=BeatThresh,"BEAT",IF(NiMy/ConsNI-1&lt;=MissThresh,"MISS","IN-LINE"))</f>
         <v>BEAT</v>
       </c>
-      <c r="L11" s="8"/>
+      <c r="L11" s="25"/>
     </row>
     <row r="13">
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
-      <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
-      <c r="L13" s="7"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
     </row>
     <row r="14">
-      <c r="B14" s="22" t="str">
+      <c r="B14" s="27" t="str">
         <f>INDEX(KpiNames,1,MATCH(SelectedSector,SectorList,0))</f>
         <v>ARR ($M)</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22" t="str">
+      <c r="C14" s="27"/>
+      <c r="D14" s="27" t="str">
         <f>INDEX(KpiNames,2,MATCH(SelectedSector,SectorList,0))</f>
         <v>Net Rev Retention (%)</v>
       </c>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22" t="str">
+      <c r="E14" s="27"/>
+      <c r="F14" s="27" t="str">
         <f>INDEX(KpiNames,3,MATCH(SelectedSector,SectorList,0))</f>
         <v>Rule of 40 (%)</v>
       </c>
-      <c r="G14" s="22"/>
-      <c r="H14" s="22" t="str">
+      <c r="G14" s="27"/>
+      <c r="H14" s="27" t="str">
         <f>INDEX(KpiNames,4,MATCH(SelectedSector,SectorList,0))</f>
         <v>Gross Margin (%)</v>
       </c>
-      <c r="I14" s="22"/>
-      <c r="J14" s="22" t="str">
+      <c r="I14" s="27"/>
+      <c r="J14" s="27" t="str">
         <f>INDEX(KpiNames,5,MATCH(SelectedSector,SectorList,0))</f>
         <v>CAC Payback (mo)</v>
       </c>
-      <c r="K14" s="22"/>
+      <c r="K14" s="27"/>
     </row>
     <row r="15">
-      <c r="B15" s="26">
+      <c r="B15" s="29">
         <f>INDEX(KpiValues,1,MATCH(SelectedSector,SectorList,0))</f>
         <v>1200</v>
       </c>
-      <c r="C15" s="26"/>
-      <c r="D15" s="26">
+      <c r="C15" s="29"/>
+      <c r="D15" s="29">
         <f>INDEX(KpiValues,2,MATCH(SelectedSector,SectorList,0))</f>
         <v>118</v>
       </c>
-      <c r="E15" s="26"/>
-      <c r="F15" s="26">
+      <c r="E15" s="29"/>
+      <c r="F15" s="29">
         <f>INDEX(KpiValues,3,MATCH(SelectedSector,SectorList,0))</f>
         <v>46</v>
       </c>
-      <c r="G15" s="26"/>
-      <c r="H15" s="26">
+      <c r="G15" s="29"/>
+      <c r="H15" s="29">
         <f>INDEX(KpiValues,4,MATCH(SelectedSector,SectorList,0))</f>
         <v>78</v>
       </c>
-      <c r="I15" s="26"/>
-      <c r="J15" s="26">
+      <c r="I15" s="29"/>
+      <c r="J15" s="29">
         <f>INDEX(KpiValues,5,MATCH(SelectedSector,SectorList,0))</f>
         <v>14</v>
       </c>
-      <c r="K15" s="26"/>
+      <c r="K15" s="29"/>
     </row>
     <row r="17">
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
-      <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
-      <c r="L17" s="7"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="6"/>
+      <c r="K17" s="6"/>
+      <c r="L17" s="6"/>
     </row>
     <row r="18">
-      <c r="B18" s="20" t="s">
+      <c r="B18" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="20" t="s">
+      <c r="C18" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="D18" s="20" t="s">
+      <c r="D18" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="E18" s="20" t="s">
+      <c r="E18" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="F18" s="20" t="s">
+      <c r="F18" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="G18" s="20" t="s">
+      <c r="G18" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="H18" s="20" t="s">
+      <c r="H18" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="I18" s="20" t="s">
+      <c r="I18" s="24" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="27">
+      <c r="B19" s="33">
         <f>Valuation!C5</f>
-        <v>11.934156378600823</v>
-      </c>
-      <c r="C19" s="27">
+        <v>14.423076923076922</v>
+      </c>
+      <c r="C19" s="33">
         <f>Valuation!C6</f>
-        <v>23.809523809523807</v>
-      </c>
-      <c r="D19" s="27">
+        <v>28.73563218390804</v>
+      </c>
+      <c r="D19" s="33">
         <f>Valuation!C7</f>
-        <v>3.2222222222222223</v>
-      </c>
-      <c r="E19" s="27">
+        <v>3.75</v>
+      </c>
+      <c r="E19" s="33">
         <f>Valuation!C8</f>
-        <v>3.3333333333333335</v>
-      </c>
-      <c r="F19" s="31">
+        <v>3.8793103448275863</v>
+      </c>
+      <c r="F19" s="41">
         <f>FairValue</f>
-        <v>97.84041184233337</v>
-      </c>
-      <c r="G19" s="31">
+        <v>45.85775303860559</v>
+      </c>
+      <c r="G19" s="41">
         <f>AvgImplied</f>
-        <v>68.7225</v>
-      </c>
-      <c r="H19" s="31">
+        <v>48.165</v>
+      </c>
+      <c r="H19" s="41">
         <f>Price</f>
         <v>45</v>
       </c>
-      <c r="I19" s="21">
+      <c r="I19" s="26">
         <f>Valuation!C35</f>
-        <v>1.1742313742740746</v>
+        <v>0.0190611786356798</v>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="7"/>
-      <c r="J21" s="7"/>
-      <c r="K21" s="7"/>
-      <c r="L21" s="7"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="6"/>
+      <c r="K21" s="6"/>
+      <c r="L21" s="6"/>
     </row>
     <row r="22">
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="D22" s="23">
+      <c r="D22" s="28">
         <f>AVERAGE(RevMy/ConsRev-1,EbitdaMy/ConsEBITDA-1,NiMy/ConsNI-1)</f>
-        <v>0.06350678733031678</v>
-      </c>
-      <c r="F22" s="4" t="s">
+        <v>0.025022844509948516</v>
+      </c>
+      <c r="F22" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="H22" s="44" t="str">
+      <c r="H22" s="45" t="str">
         <f>IF(D22&gt;=BeatThresh,"LIKELY BEAT  ▲",IF(D22&lt;=MissThresh,"LIKELY MISS  ▼","IN-LINE  ►"))</f>
         <v>LIKELY BEAT  ▲</v>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D23" s="23">
+      <c r="D23" s="28">
         <f>D22*ReactSens</f>
-        <v>0.5080542986425343</v>
-      </c>
-      <c r="F23" s="4" t="s">
+        <v>0.20018275607958813</v>
+      </c>
+      <c r="F23" s="8" t="s">
         <v>28</v>
       </c>
       <c r="H23" t="str">
@@ -1717,46 +1717,46 @@
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="10" t="s">
+      <c r="B40" s="18" t="s">
         <v>29</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="34">
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="H23:L23"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="H22:L22"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="B13:L13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="B17:L17"/>
+    <mergeCell ref="K11:L11"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="B21:L21"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="K7:L7"/>
     <mergeCell ref="K10:L10"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="B17:L17"/>
-    <mergeCell ref="B21:L21"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="C9:D9"/>
     <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="K9:L9"/>
     <mergeCell ref="J15:K15"/>
-    <mergeCell ref="H22:L22"/>
-    <mergeCell ref="H23:L23"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="K8:L8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="F6:H6"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="K11:L11"/>
-    <mergeCell ref="B13:L13"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="J14:K14"/>
   </mergeCells>
   <conditionalFormatting sqref="H22">
     <cfRule type="expression" priority="1">
@@ -1884,80 +1884,80 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
     </row>
     <row r="3">
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="F3" s="7" t="s">
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="F3" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
     </row>
     <row r="4">
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="18" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="25" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="39">
+      <c r="D6" s="40">
         <v>45</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="I6" s="11" t="s">
+      <c r="I6" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="J6" s="11" t="s">
+      <c r="J6" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="K6" s="11" t="s">
+      <c r="K6" s="9" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="D7" s="37">
+      <c r="D7" s="39">
         <v>100</v>
       </c>
       <c r="F7" t="s">
@@ -1980,10 +1980,10 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="D8" s="34">
+      <c r="D8" s="38">
         <v>-150</v>
       </c>
       <c r="F8" t="s">
@@ -2006,10 +2006,10 @@
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="30" t="s">
         <v>45</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="32">
         <v>0.21</v>
       </c>
       <c r="F9" t="s">
@@ -2032,260 +2032,260 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="D10" s="24">
+      <c r="D10" s="36">
         <v>46231</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="30" t="s">
         <v>50</v>
       </c>
-      <c r="D11" s="8" t="str">
+      <c r="D11" s="25" t="str">
         <f>SelectedSector</f>
         <v>Tech/SaaS</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
     </row>
     <row r="14">
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="D14" s="12">
-        <v>0.35</v>
+      <c r="D14" s="32">
+        <v>0.16</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="30" t="s">
         <v>53</v>
       </c>
-      <c r="D15" s="12">
-        <v>0.05</v>
+      <c r="D15" s="32">
+        <v>0.03</v>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="30" t="s">
         <v>54</v>
       </c>
-      <c r="D16" s="12">
-        <v>0.27</v>
+      <c r="D16" s="32">
+        <v>0.26</v>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="D17" s="12">
-        <v>0.14</v>
+      <c r="D17" s="32">
+        <v>0.135</v>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="D18" s="12">
+      <c r="D18" s="32">
         <v>0.85</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D19" s="25" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="30" t="s">
         <v>59</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="31">
         <f>IF(ScenarioName="Bull",1.25,IF(ScenarioName="Bear",0.7,1))</f>
         <v>1</v>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
     </row>
     <row r="23">
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="D23" s="9">
-        <v>14</v>
+      <c r="D23" s="31">
+        <v>13</v>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="30" t="s">
         <v>62</v>
       </c>
-      <c r="D24" s="9">
-        <v>24</v>
+      <c r="D24" s="31">
+        <v>22</v>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="30" t="s">
         <v>63</v>
       </c>
-      <c r="D25" s="9">
-        <v>6</v>
+      <c r="D25" s="31">
+        <v>5</v>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="30" t="s">
         <v>64</v>
       </c>
-      <c r="D26" s="9">
-        <v>7</v>
+      <c r="D26" s="31">
+        <v>5</v>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
     </row>
     <row r="29">
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="30" t="s">
         <v>66</v>
       </c>
-      <c r="D29" s="12">
+      <c r="D29" s="32">
         <v>0.042</v>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="D30" s="12">
+      <c r="D30" s="32">
         <v>0.05</v>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="30" t="s">
         <v>68</v>
       </c>
-      <c r="D31" s="33">
+      <c r="D31" s="37">
         <v>1.2</v>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="D32" s="12">
+      <c r="D32" s="32">
         <v>0.06</v>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="30" t="s">
         <v>70</v>
       </c>
-      <c r="D33" s="12">
+      <c r="D33" s="32">
         <v>0.85</v>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="30" t="s">
         <v>71</v>
       </c>
-      <c r="D34" s="12">
+      <c r="D34" s="32">
         <v>0.15</v>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="D35" s="12">
+      <c r="D35" s="32">
         <v>0.03</v>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="7" t="s">
+      <c r="B37" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
     </row>
     <row r="38">
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="D38" s="12">
+      <c r="D38" s="32">
         <v>0.02</v>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="30" t="s">
         <v>75</v>
       </c>
-      <c r="D39" s="12">
+      <c r="D39" s="32">
         <v>-0.02</v>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="30" t="s">
         <v>76</v>
       </c>
-      <c r="D40" s="9">
+      <c r="D40" s="31">
         <v>8</v>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="7" t="s">
+      <c r="B42" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="C42" s="7"/>
-      <c r="D42" s="7"/>
+      <c r="C42" s="6"/>
+      <c r="D42" s="6"/>
     </row>
     <row r="43">
-      <c r="B43" s="6" t="s">
+      <c r="B43" s="30" t="s">
         <v>78</v>
       </c>
-      <c r="D43" s="8"/>
+      <c r="D43" s="25"/>
     </row>
     <row r="44">
-      <c r="B44" s="6" t="s">
+      <c r="B44" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="D44" s="8"/>
+      <c r="D44" s="25"/>
     </row>
     <row r="45">
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="30" t="s">
         <v>80</v>
       </c>
-      <c r="D45" s="8"/>
+      <c r="D45" s="25"/>
     </row>
     <row r="46">
-      <c r="B46" s="6" t="s">
+      <c r="B46" s="30" t="s">
         <v>81</v>
       </c>
-      <c r="D46" s="8"/>
+      <c r="D46" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="F3:K3"/>
-    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B13:D13"/>
     <mergeCell ref="B37:D37"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B22:D22"/>
     <mergeCell ref="B28:D28"/>
     <mergeCell ref="B42:D42"/>
-    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="F3:K3"/>
   </mergeCells>
 </worksheet>
 </file>
@@ -2301,85 +2301,85 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
     </row>
     <row r="3">
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="16" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="4">
         <v>1000</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="4">
+        <v>1150</v>
+      </c>
+      <c r="E4" s="4">
         <v>1300</v>
       </c>
-      <c r="E4" s="1">
-        <v>1500</v>
-      </c>
     </row>
     <row r="5">
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="4">
         <v>250</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="4">
+        <v>295</v>
+      </c>
+      <c r="E5" s="4">
         <v>340</v>
       </c>
-      <c r="E5" s="1">
-        <v>400</v>
-      </c>
     </row>
     <row r="6">
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="4">
         <v>120</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="4">
+        <v>150</v>
+      </c>
+      <c r="E6" s="4">
         <v>175</v>
       </c>
-      <c r="E6" s="1">
-        <v>205</v>
-      </c>
     </row>
     <row r="7">
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="7">
         <f>C6/Shares</f>
         <v>1.2</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="7">
         <f>D6/Shares</f>
+        <v>1.5</v>
+      </c>
+      <c r="E7" s="7">
+        <f>E6/Shares</f>
         <v>1.75</v>
-      </c>
-      <c r="E7" s="3">
-        <f>E6/Shares</f>
-        <v>2.05</v>
       </c>
     </row>
   </sheetData>
@@ -2401,81 +2401,81 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
     </row>
     <row r="3">
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="16" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="4">
         <f>PriorRev*(1+RevGrowthMy*ScenarioMult)</f>
-        <v>1350</v>
-      </c>
-      <c r="D4" s="10" t="s">
+        <v>1160</v>
+      </c>
+      <c r="D4" s="18" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="4">
         <f>RevMy*EbitdaMarginMy</f>
-        <v>364.5</v>
-      </c>
-      <c r="D5" s="10" t="s">
+        <v>301.6</v>
+      </c>
+      <c r="D5" s="18" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="4">
         <f>RevMy*NiMarginMy</f>
-        <v>189.00000000000003</v>
-      </c>
-      <c r="D6" s="10" t="s">
+        <v>156.60000000000002</v>
+      </c>
+      <c r="D6" s="18" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="7">
         <f>NiMy/Shares</f>
-        <v>1.8900000000000003</v>
-      </c>
-      <c r="D7" s="10" t="s">
+        <v>1.5660000000000003</v>
+      </c>
+      <c r="D7" s="18" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="4">
         <f>EbitdaMy*(1-TaxRate)*FcfConv</f>
-        <v>244.76175000000003</v>
-      </c>
-      <c r="D8" s="10" t="s">
+        <v>202.5244</v>
+      </c>
+      <c r="D8" s="18" t="s">
         <v>99</v>
       </c>
     </row>
@@ -2497,28 +2497,28 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
     </row>
     <row r="3">
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="C3" s="7"/>
+      <c r="C3" s="6"/>
     </row>
     <row r="4">
       <c r="B4" t="s">
         <v>102</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="4">
         <f>Price*Shares+NetDebt</f>
         <v>4350</v>
       </c>
@@ -2527,100 +2527,100 @@
       <c r="B5" t="s">
         <v>103</v>
       </c>
-      <c r="C5" s="15">
+      <c r="C5" s="3">
         <f>EV/EbitdaMy</f>
-        <v>11.934156378600823</v>
+        <v>14.423076923076922</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="s">
         <v>104</v>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="3">
         <f>Price/EpsMy</f>
-        <v>23.809523809523807</v>
+        <v>28.73563218390804</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="s">
         <v>105</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="3">
         <f>EV/RevMy</f>
-        <v>3.2222222222222223</v>
+        <v>3.75</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="s">
         <v>106</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="3">
         <f>Price*Shares/RevMy</f>
-        <v>3.3333333333333335</v>
+        <v>3.8793103448275863</v>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="C10" s="7"/>
+      <c r="C10" s="6"/>
     </row>
     <row r="11">
       <c r="B11" t="s">
         <v>108</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="7">
         <f>(PeerEVEBITDA*EbitdaMy-NetDebt)/Shares</f>
-        <v>52.53</v>
+        <v>40.708</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="s">
         <v>109</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="7">
         <f>PeerPE*EpsMy</f>
-        <v>45.36000000000001</v>
+        <v>34.452000000000005</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="s">
         <v>110</v>
       </c>
-      <c r="C13" s="3">
+      <c r="C13" s="7">
         <f>(PeerEVRev*RevMy-NetDebt)/Shares</f>
-        <v>82.5</v>
+        <v>59.5</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" t="s">
         <v>111</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="7">
         <f>PeerPS*RevMy/Shares</f>
-        <v>94.5</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="C15" s="43">
+      <c r="C15" s="15">
         <f>AVERAGE(C11:C14)</f>
-        <v>68.7225</v>
+        <v>48.165</v>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="C17" s="7"/>
+      <c r="C17" s="6"/>
     </row>
     <row r="18">
       <c r="B18" t="s">
         <v>114</v>
       </c>
-      <c r="C18" s="13">
+      <c r="C18" s="1">
         <f>RiskFree+Beta*ERP</f>
         <v>0.10200000000000001</v>
       </c>
@@ -2629,388 +2629,388 @@
       <c r="B19" t="s">
         <v>115</v>
       </c>
-      <c r="C19" s="13">
+      <c r="C19" s="1">
         <f>CostDebt*(1-TaxRate)</f>
         <v>0.0474</v>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="C20" s="25">
+      <c r="C20" s="5">
         <f>WeightEquity*C18+WeightDebt*C19</f>
         <v>0.09381</v>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="7"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
     </row>
     <row r="23">
-      <c r="B23" s="30" t="s">
+      <c r="B23" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="C23" s="30">
+      <c r="C23" s="10">
         <v>1</v>
       </c>
-      <c r="D23" s="30">
+      <c r="D23" s="10">
         <v>2</v>
       </c>
-      <c r="E23" s="30">
+      <c r="E23" s="10">
         <v>3</v>
       </c>
-      <c r="F23" s="30">
+      <c r="F23" s="10">
         <v>4</v>
       </c>
-      <c r="G23" s="30">
+      <c r="G23" s="10">
         <v>5</v>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="C24" s="13">
+      <c r="C24" s="1">
         <f>MAX(RevGrowthMy*ScenarioMult,TermGrowth)</f>
-        <v>0.35</v>
-      </c>
-      <c r="D24" s="13">
+        <v>0.16</v>
+      </c>
+      <c r="D24" s="1">
         <f>MAX(C24-GrowthFade,TermGrowth)</f>
-        <v>0.3</v>
-      </c>
-      <c r="E24" s="13">
+        <v>0.13</v>
+      </c>
+      <c r="E24" s="1">
         <f>MAX(D24-GrowthFade,TermGrowth)</f>
-        <v>0.25</v>
-      </c>
-      <c r="F24" s="13">
+        <v>0.1</v>
+      </c>
+      <c r="F24" s="1">
         <f>MAX(E24-GrowthFade,TermGrowth)</f>
-        <v>0.2</v>
-      </c>
-      <c r="G24" s="13">
+        <v>0.07</v>
+      </c>
+      <c r="G24" s="1">
         <f>MAX(F24-GrowthFade,TermGrowth)</f>
-        <v>0.15000000000000002</v>
+        <v>0.04000000000000001</v>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="C25" s="1">
+      <c r="C25" s="4">
         <f>RevMy*(1+C24)</f>
-        <v>1822.5000000000002</v>
-      </c>
-      <c r="D25" s="1">
+        <v>1345.6</v>
+      </c>
+      <c r="D25" s="4">
         <f>C25*(1+D24)</f>
-        <v>2369.2500000000005</v>
-      </c>
-      <c r="E25" s="1">
+        <v>1520.5279999999998</v>
+      </c>
+      <c r="E25" s="4">
         <f>D25*(1+E24)</f>
-        <v>2961.5625000000005</v>
-      </c>
-      <c r="F25" s="1">
+        <v>1672.5808</v>
+      </c>
+      <c r="F25" s="4">
         <f>E25*(1+F24)</f>
-        <v>3553.8750000000005</v>
-      </c>
-      <c r="G25" s="1">
+        <v>1789.661456</v>
+      </c>
+      <c r="G25" s="4">
         <f>F25*(1+G24)</f>
-        <v>4086.95625</v>
+        <v>1861.24791424</v>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C26" s="1">
+      <c r="C26" s="4">
         <f>C25*EbitdaMarginMy</f>
-        <v>492.0750000000001</v>
-      </c>
-      <c r="D26" s="1">
+        <v>349.856</v>
+      </c>
+      <c r="D26" s="4">
         <f>D25*EbitdaMarginMy</f>
-        <v>639.6975000000002</v>
-      </c>
-      <c r="E26" s="1">
+        <v>395.33727999999996</v>
+      </c>
+      <c r="E26" s="4">
         <f>E25*EbitdaMarginMy</f>
-        <v>799.6218750000002</v>
-      </c>
-      <c r="F26" s="1">
+        <v>434.871008</v>
+      </c>
+      <c r="F26" s="4">
         <f>F25*EbitdaMarginMy</f>
-        <v>959.5462500000002</v>
-      </c>
-      <c r="G26" s="1">
+        <v>465.31197856</v>
+      </c>
+      <c r="G26" s="4">
         <f>G25*EbitdaMarginMy</f>
-        <v>1103.4781875</v>
+        <v>483.9244577024</v>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="C27" s="1">
+      <c r="C27" s="4">
         <f>C26*(1-TaxRate)*FcfConv</f>
-        <v>330.42836250000005</v>
-      </c>
-      <c r="D27" s="1">
+        <v>234.92830399999997</v>
+      </c>
+      <c r="D27" s="4">
         <f>D26*(1-TaxRate)*FcfConv</f>
-        <v>429.55687125000014</v>
-      </c>
-      <c r="E27" s="1">
+        <v>265.46898351999994</v>
+      </c>
+      <c r="E27" s="4">
         <f>E26*(1-TaxRate)*FcfConv</f>
-        <v>536.9460890625002</v>
-      </c>
-      <c r="F27" s="1">
+        <v>292.015881872</v>
+      </c>
+      <c r="F27" s="4">
         <f>F26*(1-TaxRate)*FcfConv</f>
-        <v>644.3353068750001</v>
-      </c>
-      <c r="G27" s="1">
+        <v>312.45699360304</v>
+      </c>
+      <c r="G27" s="4">
         <f>G26*(1-TaxRate)*FcfConv</f>
-        <v>740.98560290625</v>
+        <v>324.95527334716155</v>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="s">
         <v>121</v>
       </c>
-      <c r="C29" s="1">
+      <c r="C29" s="4">
         <f>NPV(WACC,C27:G27)</f>
-        <v>1994.8249669682004</v>
+        <v>1085.6378864760316</v>
       </c>
     </row>
     <row r="30">
       <c r="B30" t="s">
         <v>122</v>
       </c>
-      <c r="C30" s="1">
+      <c r="C30" s="4">
         <f>G27*(1+TermGrowth)/(WACC-TermGrowth)</f>
-        <v>11960.74551000529</v>
+        <v>5245.320977081592</v>
       </c>
     </row>
     <row r="31">
       <c r="B31" t="s">
         <v>123</v>
       </c>
-      <c r="C31" s="1">
+      <c r="C31" s="4">
         <f>C30/(1+WACC)^5</f>
-        <v>7639.216217265135</v>
+        <v>3350.137417384527</v>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="C32" s="1">
+      <c r="C32" s="4">
         <f>C29+C31</f>
-        <v>9634.041184233336</v>
+        <v>4435.775303860559</v>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="C33" s="1">
+      <c r="C33" s="4">
         <f>C32-NetDebt</f>
-        <v>9784.041184233336</v>
+        <v>4585.775303860559</v>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="C34" s="38">
+      <c r="C34" s="11">
         <f>C33/Shares</f>
-        <v>97.84041184233337</v>
+        <v>45.85775303860559</v>
       </c>
     </row>
     <row r="35">
       <c r="B35" t="s">
         <v>127</v>
       </c>
-      <c r="C35" s="41">
+      <c r="C35" s="13">
         <f>FairValue/Price-1</f>
-        <v>1.1742313742740746</v>
+        <v>0.0190611786356798</v>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="7" t="s">
+      <c r="B37" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
-      <c r="E37" s="7"/>
-      <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
-      <c r="H37" s="7"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
     </row>
     <row r="38">
-      <c r="B38" s="42" t="s">
+      <c r="B38" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="C38" s="42">
+      <c r="C38" s="14">
         <f>TermGrowth+-0.01</f>
         <v>0.019999999999999997</v>
       </c>
-      <c r="D38" s="42">
+      <c r="D38" s="14">
         <f>TermGrowth+-0.005</f>
         <v>0.024999999999999998</v>
       </c>
-      <c r="E38" s="42">
+      <c r="E38" s="14">
         <f>TermGrowth+0</f>
         <v>0.03</v>
       </c>
-      <c r="F38" s="42">
+      <c r="F38" s="14">
         <f>TermGrowth+0.005</f>
         <v>0.034999999999999996</v>
       </c>
-      <c r="G38" s="42">
+      <c r="G38" s="14">
         <f>TermGrowth+0.01</f>
         <v>0.04</v>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="25">
+      <c r="B39" s="5">
         <f>WACC+-0.01</f>
         <v>0.08381000000000001</v>
       </c>
-      <c r="C39" s="14">
+      <c r="C39" s="2">
         <f>(NPV($B39,$C$27:$G$27)+($G$27*(1+C$38)/($B39-C$38))/(1+$B39)^5-NetDebt)/Shares</f>
-        <v>101.25366500404992</v>
-      </c>
-      <c r="D39" s="14">
+        <v>47.39403874756321</v>
+      </c>
+      <c r="D39" s="2">
         <f>(NPV($B39,$C$27:$G$27)+($G$27*(1+D$38)/($B39-D$38))/(1+$B39)^5-NetDebt)/Shares</f>
-        <v>108.40895491829501</v>
-      </c>
-      <c r="E39" s="14">
+        <v>50.53195287280684</v>
+      </c>
+      <c r="E39" s="2">
         <f>(NPV($B39,$C$27:$G$27)+($G$27*(1+E$38)/($B39-E$38))/(1+$B39)^5-NetDebt)/Shares</f>
-        <v>116.89397720835223</v>
-      </c>
-      <c r="F39" s="14">
+        <v>54.253014020024786</v>
+      </c>
+      <c r="F39" s="2">
         <f>(NPV($B39,$C$27:$G$27)+($G$27*(1+F$38)/($B39-F$38))/(1+$B39)^5-NetDebt)/Shares</f>
-        <v>127.1173773492714</v>
-      </c>
-      <c r="G39" s="14">
+        <v>58.73643147685507</v>
+      </c>
+      <c r="G39" s="2">
         <f>(NPV($B39,$C$27:$G$27)+($G$27*(1+G$38)/($B39-G$38))/(1+$B39)^5-NetDebt)/Shares</f>
-        <v>139.6743543313043</v>
+        <v>64.24322657733528</v>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="25">
+      <c r="B40" s="5">
         <f>WACC+-0.005</f>
         <v>0.08881</v>
       </c>
-      <c r="C40" s="14">
+      <c r="C40" s="2">
         <f>(NPV($B40,$C$27:$G$27)+($G$27*(1+C$38)/($B40-C$38))/(1+$B40)^5-NetDebt)/Shares</f>
-        <v>93.52395956795796</v>
-      </c>
-      <c r="D40" s="14">
+        <v>43.98434802278164</v>
+      </c>
+      <c r="D40" s="2">
         <f>(NPV($B40,$C$27:$G$27)+($G$27*(1+D$38)/($B40-D$38))/(1+$B40)^5-NetDebt)/Shares</f>
-        <v>99.5278266375593</v>
-      </c>
-      <c r="E40" s="14">
+        <v>46.61731181734158</v>
+      </c>
+      <c r="E40" s="2">
         <f>(NPV($B40,$C$27:$G$27)+($G$27*(1+E$38)/($B40-E$38))/(1+$B40)^5-NetDebt)/Shares</f>
-        <v>106.55258591420052</v>
-      </c>
-      <c r="F40" s="14">
+        <v>49.69798242954478</v>
+      </c>
+      <c r="F40" s="2">
         <f>(NPV($B40,$C$27:$G$27)+($G$27*(1+F$38)/($B40-F$38))/(1+$B40)^5-NetDebt)/Shares</f>
-        <v>114.88281987522028</v>
-      </c>
-      <c r="G40" s="14">
+        <v>53.35116198287474</v>
+      </c>
+      <c r="G40" s="2">
         <f>(NPV($B40,$C$27:$G$27)+($G$27*(1+G$38)/($B40-G$38))/(1+$B40)^5-NetDebt)/Shares</f>
-        <v>124.91971926566436</v>
+        <v>57.75279053299431</v>
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="25">
+      <c r="B41" s="5">
         <f>WACC+0</f>
         <v>0.09381</v>
       </c>
-      <c r="C41" s="14">
+      <c r="C41" s="2">
         <f>(NPV($B41,$C$27:$G$27)+($G$27*(1+C$38)/($B41-C$38))/(1+$B41)^5-NetDebt)/Shares</f>
-        <v>86.84938516979999</v>
-      </c>
-      <c r="D41" s="14">
+        <v>41.03769707161954</v>
+      </c>
+      <c r="D41" s="2">
         <f>(NPV($B41,$C$27:$G$27)+($G$27*(1+D$38)/($B41-D$38))/(1+$B41)^5-NetDebt)/Shares</f>
-        <v>91.94557331087216</v>
-      </c>
-      <c r="E41" s="14">
+        <v>43.27260312635998</v>
+      </c>
+      <c r="E41" s="2">
         <f>(NPV($B41,$C$27:$G$27)+($G$27*(1+E$38)/($B41-E$38))/(1+$B41)^5-NetDebt)/Shares</f>
-        <v>97.84041184233337</v>
-      </c>
-      <c r="F41" s="14">
+        <v>45.85775303860559</v>
+      </c>
+      <c r="F41" s="2">
         <f>(NPV($B41,$C$27:$G$27)+($G$27*(1+F$38)/($B41-F$38))/(1+$B41)^5-NetDebt)/Shares</f>
-        <v>104.73760346535397</v>
-      </c>
-      <c r="G41" s="14">
+        <v>48.882479538548104</v>
+      </c>
+      <c r="G41" s="2">
         <f>(NPV($B41,$C$27:$G$27)+($G$27*(1+G$38)/($B41-G$38))/(1+$B41)^5-NetDebt)/Shares</f>
-        <v>112.91656271948791</v>
+        <v>52.469318378193755</v>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="25">
+      <c r="B42" s="5">
         <f>WACC+0.005</f>
         <v>0.09881000000000001</v>
       </c>
-      <c r="C42" s="14">
+      <c r="C42" s="2">
         <f>(NPV($B42,$C$27:$G$27)+($G$27*(1+C$38)/($B42-C$38))/(1+$B42)^5-NetDebt)/Shares</f>
-        <v>81.02894602071116</v>
-      </c>
-      <c r="D42" s="14">
+        <v>38.465933352713236</v>
+      </c>
+      <c r="D42" s="2">
         <f>(NPV($B42,$C$27:$G$27)+($G$27*(1+D$38)/($B42-D$38))/(1+$B42)^5-NetDebt)/Shares</f>
-        <v>85.39805450871</v>
-      </c>
-      <c r="E42" s="14">
+        <v>40.381982514036416</v>
+      </c>
+      <c r="E42" s="2">
         <f>(NPV($B42,$C$27:$G$27)+($G$27*(1+E$38)/($B42-E$38))/(1+$B42)^5-NetDebt)/Shares</f>
-        <v>90.40211554546619</v>
-      </c>
-      <c r="F42" s="14">
+        <v>42.576486719876854</v>
+      </c>
+      <c r="F42" s="2">
         <f>(NPV($B42,$C$27:$G$27)+($G$27*(1+F$38)/($B42-F$38))/(1+$B42)^5-NetDebt)/Shares</f>
-        <v>96.19038925057464</v>
-      </c>
-      <c r="G42" s="14">
+        <v>45.114903197436526</v>
+      </c>
+      <c r="G42" s="2">
         <f>(NPV($B42,$C$27:$G$27)+($G$27*(1+G$38)/($B42-G$38))/(1+$B42)^5-NetDebt)/Shares</f>
-        <v>102.96289585911936</v>
+        <v>48.08494975109885</v>
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="25">
+      <c r="B43" s="5">
         <f>WACC+0.01</f>
         <v>0.10381</v>
       </c>
-      <c r="C43" s="14">
+      <c r="C43" s="2">
         <f>(NPV($B43,$C$27:$G$27)+($G$27*(1+C$38)/($B43-C$38))/(1+$B43)^5-NetDebt)/Shares</f>
-        <v>75.90961553246989</v>
-      </c>
-      <c r="D43" s="14">
+        <v>36.201941148015415</v>
+      </c>
+      <c r="D43" s="2">
         <f>(NPV($B43,$C$27:$G$27)+($G$27*(1+D$38)/($B43-D$38))/(1+$B43)^5-NetDebt)/Shares</f>
-        <v>79.68816671232037</v>
-      </c>
-      <c r="E43" s="14">
+        <v>37.85900456016365</v>
+      </c>
+      <c r="E43" s="2">
         <f>(NPV($B43,$C$27:$G$27)+($G$27*(1+E$38)/($B43-E$38))/(1+$B43)^5-NetDebt)/Shares</f>
-        <v>83.97864732989616</v>
-      </c>
-      <c r="F43" s="14">
+        <v>39.74057188941638</v>
+      </c>
+      <c r="F43" s="2">
         <f>(NPV($B43,$C$27:$G$27)+($G$27*(1+F$38)/($B43-F$38))/(1+$B43)^5-NetDebt)/Shares</f>
-        <v>88.89265368756432</v>
-      </c>
-      <c r="G43" s="14">
+        <v>41.895583097357196</v>
+      </c>
+      <c r="G43" s="2">
         <f>(NPV($B43,$C$27:$G$27)+($G$27*(1+G$38)/($B43-G$38))/(1+$B43)^5-NetDebt)/Shares</f>
-        <v>94.57675977218254</v>
+        <v>44.38831742204161</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="B22:H22"/>
+    <mergeCell ref="B37:H37"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="B22:H22"/>
-    <mergeCell ref="B10:C10"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B37:H37"/>
+    <mergeCell ref="B10:C10"/>
   </mergeCells>
   <conditionalFormatting sqref="C39:G43">
     <cfRule type="colorScale" priority="1">
@@ -3038,37 +3038,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
     </row>
     <row r="3">
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="16" t="s">
         <v>132</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="16" t="s">
         <v>133</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="16" t="s">
         <v>134</v>
       </c>
     </row>
@@ -3076,111 +3076,111 @@
       <c r="B4" t="s">
         <v>58</v>
       </c>
-      <c r="C4" s="13">
+      <c r="C4" s="1">
         <f>RevGrowthMy</f>
-        <v>0.35</v>
-      </c>
-      <c r="D4" s="13">
+        <v>0.16</v>
+      </c>
+      <c r="D4" s="1">
         <f>EbitdaMarginMy</f>
-        <v>0.27</v>
-      </c>
-      <c r="E4" s="1">
+        <v>0.26</v>
+      </c>
+      <c r="E4" s="4">
         <f>PriorRev*(1+C4)</f>
-        <v>1350</v>
-      </c>
-      <c r="F4" s="1">
+        <v>1160</v>
+      </c>
+      <c r="F4" s="4">
         <f>E4*D4</f>
-        <v>364.5</v>
-      </c>
-      <c r="G4" s="3">
+        <v>301.6</v>
+      </c>
+      <c r="G4" s="7">
         <f>(PeerEVEBITDA*F4-NetDebt)/Shares</f>
-        <v>52.53</v>
-      </c>
-      <c r="H4" s="13">
+        <v>40.708</v>
+      </c>
+      <c r="H4" s="1">
         <f>G4/Price-1</f>
-        <v>0.16733333333333333</v>
+        <v>-0.09537777777777778</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="s">
         <v>135</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="1">
         <f>RevGrowthMy*1.25</f>
-        <v>0.4375</v>
-      </c>
-      <c r="D5" s="13">
+        <v>0.2</v>
+      </c>
+      <c r="D5" s="1">
         <f>EbitdaMarginMy+0.03</f>
-        <v>0.30000000000000004</v>
-      </c>
-      <c r="E5" s="1">
+        <v>0.29000000000000004</v>
+      </c>
+      <c r="E5" s="4">
         <f>PriorRev*(1+C5)</f>
-        <v>1437.5</v>
-      </c>
-      <c r="F5" s="1">
+        <v>1200</v>
+      </c>
+      <c r="F5" s="4">
         <f>E5*D5</f>
-        <v>431.25000000000006</v>
-      </c>
-      <c r="G5" s="3">
+        <v>348.00000000000006</v>
+      </c>
+      <c r="G5" s="7">
         <f>(PeerEVEBITDA*F5-NetDebt)/Shares</f>
-        <v>61.87500000000001</v>
-      </c>
-      <c r="H5" s="13">
+        <v>46.74000000000001</v>
+      </c>
+      <c r="H5" s="1">
         <f>G5/Price-1</f>
-        <v>0.3750000000000002</v>
+        <v>0.03866666666666685</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="s">
         <v>136</v>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="1">
         <f>RevGrowthMy*0.7</f>
-        <v>0.24499999999999997</v>
-      </c>
-      <c r="D6" s="13">
+        <v>0.11199999999999999</v>
+      </c>
+      <c r="D6" s="1">
         <f>EbitdaMarginMy-0.04</f>
-        <v>0.23</v>
-      </c>
-      <c r="E6" s="1">
+        <v>0.22</v>
+      </c>
+      <c r="E6" s="4">
         <f>PriorRev*(1+C6)</f>
-        <v>1244.9999999999998</v>
-      </c>
-      <c r="F6" s="1">
+        <v>1112</v>
+      </c>
+      <c r="F6" s="4">
         <f>E6*D6</f>
-        <v>286.34999999999997</v>
-      </c>
-      <c r="G6" s="3">
+        <v>244.64000000000001</v>
+      </c>
+      <c r="G6" s="7">
         <f>(PeerEVEBITDA*F6-NetDebt)/Shares</f>
-        <v>41.589</v>
-      </c>
-      <c r="H6" s="13">
+        <v>33.303200000000004</v>
+      </c>
+      <c r="H6" s="1">
         <f>G6/Price-1</f>
-        <v>-0.07579999999999998</v>
+        <v>-0.25992888888888876</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
     </row>
     <row r="9">
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="9" t="s">
         <v>141</v>
       </c>
     </row>
@@ -3188,66 +3188,66 @@
       <c r="B10" t="s">
         <v>142</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="7">
         <f>(PeerEVEBITDA*(PriorRev*(1+RevGrowthMy*0.8)*EbitdaMarginMy)-NetDebt)/Shares</f>
-        <v>49.88400000000001</v>
-      </c>
-      <c r="D10" s="3">
+        <v>39.626400000000004</v>
+      </c>
+      <c r="D10" s="7">
         <f>(PeerEVEBITDA*(PriorRev*(1+RevGrowthMy*1.2)*EbitdaMarginMy)-NetDebt)/Shares</f>
-        <v>55.176</v>
-      </c>
-      <c r="E10" s="3">
+        <v>41.7896</v>
+      </c>
+      <c r="E10" s="7">
         <f>ABS(D10-C10)</f>
-        <v>5.2919999999999945</v>
+        <v>2.1631999999999962</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" t="s">
         <v>54</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="7">
         <f>(PeerEVEBITDA*(PriorRev*(1+RevGrowthMy)*EbitdaMarginMy*0.8)-NetDebt)/Shares</f>
-        <v>42.324000000000005</v>
-      </c>
-      <c r="D11" s="3">
+        <v>32.866400000000006</v>
+      </c>
+      <c r="D11" s="7">
         <f>(PeerEVEBITDA*(PriorRev*(1+RevGrowthMy)*EbitdaMarginMy*1.2)-NetDebt)/Shares</f>
-        <v>62.736</v>
-      </c>
-      <c r="E11" s="3">
+        <v>48.5496</v>
+      </c>
+      <c r="E11" s="7">
         <f>ABS(D11-C11)</f>
-        <v>20.411999999999992</v>
+        <v>15.683199999999992</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="s">
         <v>61</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="7">
         <f>(PeerEVEBITDA*0.8*(PriorRev*(1+RevGrowthMy)*EbitdaMarginMy)-NetDebt)/Shares</f>
-        <v>42.324000000000005</v>
-      </c>
-      <c r="D12" s="3">
+        <v>32.866400000000006</v>
+      </c>
+      <c r="D12" s="7">
         <f>(PeerEVEBITDA*1.2*(PriorRev*(1+RevGrowthMy)*EbitdaMarginMy)-NetDebt)/Shares</f>
-        <v>62.736000000000004</v>
-      </c>
-      <c r="E12" s="3">
+        <v>48.5496</v>
+      </c>
+      <c r="E12" s="7">
         <f>ABS(D12-C12)</f>
-        <v>20.412</v>
+        <v>15.683199999999992</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="s">
         <v>143</v>
       </c>
-      <c r="C13" s="3">
+      <c r="C13" s="7">
         <f>(PeerEVEBITDA*(PriorRev*(1+RevGrowthMy)*EbitdaMarginMy)-NetDebt*1.2)/Shares</f>
-        <v>52.83</v>
-      </c>
-      <c r="D13" s="3">
+        <v>41.008</v>
+      </c>
+      <c r="D13" s="7">
         <f>(PeerEVEBITDA*(PriorRev*(1+RevGrowthMy)*EbitdaMarginMy)-NetDebt*0.8)/Shares</f>
-        <v>52.23</v>
-      </c>
-      <c r="E13" s="3">
+        <v>40.408</v>
+      </c>
+      <c r="E13" s="7">
         <f>ABS(D13-C13)</f>
         <v>0.6000000000000014</v>
       </c>
@@ -3256,17 +3256,17 @@
       <c r="B14" t="s">
         <v>144</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="7">
         <f>(PeerEVEBITDA*(PriorRev*(1+RevGrowthMy)*EbitdaMarginMy)-NetDebt)/Shares*1.2</f>
-        <v>63.036</v>
-      </c>
-      <c r="D14" s="3">
+        <v>48.849599999999995</v>
+      </c>
+      <c r="D14" s="7">
         <f>(PeerEVEBITDA*(PriorRev*(1+RevGrowthMy)*EbitdaMarginMy)-NetDebt)/Shares*0.8</f>
-        <v>42.024</v>
-      </c>
-      <c r="E14" s="3">
+        <v>32.5664</v>
+      </c>
+      <c r="E14" s="7">
         <f>ABS(D14-C14)</f>
-        <v>21.012</v>
+        <v>16.283199999999994</v>
       </c>
     </row>
   </sheetData>
@@ -3295,23 +3295,23 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="16" t="s">
         <v>147</v>
       </c>
     </row>
@@ -3319,46 +3319,46 @@
       <c r="A4" t="s">
         <v>87</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="4">
         <f>ConsRev</f>
-        <v>1300</v>
-      </c>
-      <c r="C4" s="1">
+        <v>1150</v>
+      </c>
+      <c r="C4" s="4">
         <f>RevMy</f>
-        <v>1350</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
         <v>88</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="4">
         <f>ConsEBITDA</f>
-        <v>340</v>
-      </c>
-      <c r="C5" s="1">
+        <v>295</v>
+      </c>
+      <c r="C5" s="4">
         <f>EbitdaMy</f>
-        <v>364.5</v>
+        <v>301.6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
         <v>89</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="4">
         <f>ConsNI</f>
-        <v>175</v>
-      </c>
-      <c r="C6" s="1">
+        <v>150</v>
+      </c>
+      <c r="C6" s="4">
         <f>NiMy</f>
-        <v>189.00000000000003</v>
+        <v>156.60000000000002</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="16" t="s">
         <v>149</v>
       </c>
     </row>
@@ -3367,7 +3367,7 @@
         <f>INDEX(KpiNames,1,MATCH(SelectedSector,SectorList,0))</f>
         <v>ARR ($M)</v>
       </c>
-      <c r="B10" s="40">
+      <c r="B10" s="17">
         <f>INDEX(KpiValues,1,MATCH(SelectedSector,SectorList,0))</f>
         <v>1200</v>
       </c>
@@ -3377,7 +3377,7 @@
         <f>INDEX(KpiNames,2,MATCH(SelectedSector,SectorList,0))</f>
         <v>Net Rev Retention (%)</v>
       </c>
-      <c r="B11" s="40">
+      <c r="B11" s="17">
         <f>INDEX(KpiValues,2,MATCH(SelectedSector,SectorList,0))</f>
         <v>118</v>
       </c>
@@ -3387,7 +3387,7 @@
         <f>INDEX(KpiNames,3,MATCH(SelectedSector,SectorList,0))</f>
         <v>Rule of 40 (%)</v>
       </c>
-      <c r="B12" s="40">
+      <c r="B12" s="17">
         <f>INDEX(KpiValues,3,MATCH(SelectedSector,SectorList,0))</f>
         <v>46</v>
       </c>
@@ -3397,7 +3397,7 @@
         <f>INDEX(KpiNames,4,MATCH(SelectedSector,SectorList,0))</f>
         <v>Gross Margin (%)</v>
       </c>
-      <c r="B13" s="40">
+      <c r="B13" s="17">
         <f>INDEX(KpiValues,4,MATCH(SelectedSector,SectorList,0))</f>
         <v>78</v>
       </c>
@@ -3407,16 +3407,16 @@
         <f>INDEX(KpiNames,5,MATCH(SelectedSector,SectorList,0))</f>
         <v>CAC Payback (mo)</v>
       </c>
-      <c r="B14" s="40">
+      <c r="B14" s="17">
         <f>INDEX(KpiValues,5,MATCH(SelectedSector,SectorList,0))</f>
         <v>14</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="16" t="s">
         <v>149</v>
       </c>
     </row>
@@ -3424,36 +3424,36 @@
       <c r="A18" t="s">
         <v>151</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B18" s="4">
         <f>ConsNI</f>
-        <v>175</v>
+        <v>150</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
         <v>152</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B19" s="4">
         <f>(RevMy-ConsRev)*NiMarginMy</f>
-        <v>7.000000000000001</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
         <v>153</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B20" s="4">
         <f>NiMy-ConsNI-((RevMy-ConsRev)*NiMarginMy)</f>
-        <v>7.0000000000000275</v>
+        <v>5.250000000000023</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
         <v>154</v>
       </c>
-      <c r="B21" s="1">
+      <c r="B21" s="4">
         <f>NiMy</f>
-        <v>189.00000000000003</v>
+        <v>156.60000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -3473,46 +3473,46 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="20" t="s">
         <v>156</v>
       </c>
-      <c r="C3" s="30" t="s">
+      <c r="C3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="30" t="s">
+      <c r="D3" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="E3" s="30" t="s">
+      <c r="E3" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="F3" s="30" t="s">
+      <c r="F3" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="G3" s="30" t="s">
+      <c r="G3" s="10" t="s">
         <v>158</v>
       </c>
-      <c r="H3" s="30" t="s">
+      <c r="H3" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="I3" s="30" t="s">
+      <c r="I3" s="10" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17"/>
+      <c r="A4" s="20"/>
       <c r="C4" t="s">
         <v>161</v>
       </c>
@@ -3536,7 +3536,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17"/>
+      <c r="A5" s="20"/>
       <c r="C5" t="s">
         <v>168</v>
       </c>
@@ -3560,7 +3560,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17"/>
+      <c r="A6" s="20"/>
       <c r="C6" t="s">
         <v>174</v>
       </c>
@@ -3584,7 +3584,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17"/>
+      <c r="A7" s="20"/>
       <c r="C7" t="s">
         <v>169</v>
       </c>
@@ -3608,7 +3608,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17"/>
+      <c r="A8" s="20"/>
       <c r="C8" t="s">
         <v>185</v>
       </c>
@@ -3632,148 +3632,148 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="20" t="s">
         <v>191</v>
       </c>
-      <c r="C10" s="30" t="s">
+      <c r="C10" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D10" s="30" t="s">
+      <c r="D10" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="E10" s="30" t="s">
+      <c r="E10" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="F10" s="30" t="s">
+      <c r="F10" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="G10" s="30" t="s">
+      <c r="G10" s="10" t="s">
         <v>158</v>
       </c>
-      <c r="H10" s="30" t="s">
+      <c r="H10" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="I10" s="30" t="s">
+      <c r="I10" s="10" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17"/>
-      <c r="C11" s="46">
+      <c r="A11" s="20"/>
+      <c r="C11" s="19">
         <v>1200</v>
       </c>
-      <c r="D11" s="46">
+      <c r="D11" s="19">
         <v>4.5</v>
       </c>
-      <c r="E11" s="46">
+      <c r="E11" s="19">
         <v>22</v>
       </c>
-      <c r="F11" s="46">
+      <c r="F11" s="19">
         <v>1.08</v>
       </c>
-      <c r="G11" s="46">
+      <c r="G11" s="19">
         <v>3.2</v>
       </c>
-      <c r="H11" s="46">
+      <c r="H11" s="19">
         <v>520</v>
       </c>
-      <c r="I11" s="46">
+      <c r="I11" s="19">
         <v>12</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17"/>
-      <c r="C12" s="46">
+      <c r="A12" s="20"/>
+      <c r="C12" s="19">
         <v>118</v>
       </c>
-      <c r="D12" s="46">
+      <c r="D12" s="19">
         <v>42</v>
       </c>
-      <c r="E12" s="46">
+      <c r="E12" s="19">
         <v>12</v>
       </c>
-      <c r="F12" s="46">
+      <c r="F12" s="19">
         <v>84</v>
       </c>
-      <c r="G12" s="46">
+      <c r="G12" s="19">
         <v>58</v>
       </c>
-      <c r="H12" s="46">
+      <c r="H12" s="19">
         <v>68</v>
       </c>
-      <c r="I12" s="46">
+      <c r="I12" s="19">
         <v>55</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="17"/>
-      <c r="C13" s="46">
+      <c r="A13" s="20"/>
+      <c r="C13" s="19">
         <v>46</v>
       </c>
-      <c r="D13" s="46">
+      <c r="D13" s="19">
         <v>5.2</v>
       </c>
-      <c r="E13" s="46">
+      <c r="E13" s="19">
         <v>340</v>
       </c>
-      <c r="F13" s="46">
+      <c r="F13" s="19">
         <v>2300</v>
       </c>
-      <c r="G13" s="46">
+      <c r="G13" s="19">
         <v>13.5</v>
       </c>
-      <c r="H13" s="46">
+      <c r="H13" s="19">
         <v>12.5</v>
       </c>
-      <c r="I13" s="46">
+      <c r="I13" s="19">
         <v>20</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="17"/>
-      <c r="C14" s="46">
+      <c r="A14" s="20"/>
+      <c r="C14" s="19">
         <v>78</v>
       </c>
-      <c r="D14" s="46">
+      <c r="D14" s="19">
         <v>1450</v>
       </c>
-      <c r="E14" s="46">
+      <c r="E14" s="19">
         <v>74</v>
       </c>
-      <c r="F14" s="46">
+      <c r="F14" s="19">
         <v>16</v>
       </c>
-      <c r="G14" s="46">
+      <c r="G14" s="19">
         <v>12.2</v>
       </c>
-      <c r="H14" s="46">
+      <c r="H14" s="19">
         <v>9.4</v>
       </c>
-      <c r="I14" s="46">
+      <c r="I14" s="19">
         <v>18</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="17"/>
-      <c r="C15" s="46">
+      <c r="A15" s="20"/>
+      <c r="C15" s="19">
         <v>14</v>
       </c>
-      <c r="D15" s="46">
+      <c r="D15" s="19">
         <v>31</v>
       </c>
-      <c r="E15" s="46">
+      <c r="E15" s="19">
         <v>28</v>
       </c>
-      <c r="F15" s="46">
+      <c r="F15" s="19">
         <v>13</v>
       </c>
-      <c r="G15" s="46">
+      <c r="G15" s="19">
         <v>7</v>
       </c>
-      <c r="H15" s="46">
+      <c r="H15" s="19">
         <v>11</v>
       </c>
-      <c r="I15" s="46">
+      <c r="I15" s="19">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Cell-by-cell audit fixes: shares pull + Dashboard header formats
Systematic per-tab/per-cell audit (value, formula, number-format, type) of all
8 tabs. Findings + fixes:
- SHARES (CapIQ) now derived as MarketCap/Price: =CIQ(Ticker,"IQ_MARKETCAP")
  *1e-6/Price. Robust to CapIQ's share-count unit convention (the likely cause
  of the wrong pull) and guaranteed in millions to match the (M) label; EV then
  resolves to MktCap+NetDebt as expected.
- Dashboard header Price (J3) and Shares (J4) were unformatted — the formats had
  been applied to the empty K3/K4. Now J3=$#,##0.00, J4=#,##0, F4=date.
- Inputs 'Load Example Template' value columns (I7:K9) now formatted ($/#/$).
- Verified everything else pulls/formats correctly across Dashboard, Inputs,
  Consensus, MyModel, Valuation (incl. full DCF + sensitivity grid), Scenarios,
  Charts, SectorKPIs; large-number (Apple-scale) handling sane (EV $2.95T,
  EV/EBITDA 25.6x).
</commit_message>
<xml_diff>
--- a/Sector_Consensus_vs_My_Model.xlsx
+++ b/Sector_Consensus_vs_My_Model.xlsx
@@ -651,12 +651,12 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="7">
     <numFmt numFmtId="164" formatCode="$#,##0.0"/>
-    <numFmt numFmtId="165" formatCode="$#,##0.00"/>
-    <numFmt numFmtId="166" formatCode="0.0&quot;x&quot;"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
-    <numFmt numFmtId="168" formatCode="MMM D, YYYY"/>
-    <numFmt numFmtId="169" formatCode="#,##0.0"/>
-    <numFmt numFmtId="170" formatCode="#,##0"/>
+    <numFmt numFmtId="168" formatCode="0.0&quot;x&quot;"/>
+    <numFmt numFmtId="169" formatCode="#,##0"/>
+    <numFmt numFmtId="170" formatCode="MMM D, YYYY"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -673,18 +673,22 @@
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
     </font>
     <font>
-      <color rgb="FF1A1A1A"/>
+      <b/>
+      <color rgb="FF2E5C9A"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <color rgb="FF1A1A1A"/>
     </font>
     <font>
       <i/>
@@ -696,7 +700,7 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF2E5C9A"/>
+      <sz val="14"/>
     </font>
     <font>
       <b/>
@@ -705,7 +709,10 @@
     </font>
     <font>
       <b/>
-      <sz val="14"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="0"/>
     </font>
     <font>
       <b/>
@@ -713,15 +720,8 @@
       <color rgb="FFFFFFFF"/>
     </font>
     <font>
-      <b val="0"/>
-    </font>
-    <font>
       <b/>
       <color rgb="FF9C6500"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
     </font>
   </fonts>
   <fills count="9">
@@ -745,14 +745,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F6FC"/>
-        <bgColor rgb="FFF2F6FC"/>
+        <fgColor rgb="FFD9E1F2"/>
+        <bgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9E1F2"/>
-        <bgColor rgb="FFD9E1F2"/>
+        <fgColor rgb="FFF2F6FC"/>
+        <bgColor rgb="FFF2F6FC"/>
       </patternFill>
     </fill>
     <fill>
@@ -794,87 +794,88 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="170" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="12" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1428,400 +1429,397 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
     </row>
     <row r="3">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="8" t="s">
         <v>1</v>
       </c>
       <c r="B3" t="str">
         <f>Inputs!D4</f>
         <v>Nimbus Cloud Inc</v>
       </c>
-      <c r="E3" s="25" t="s">
+      <c r="E3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="44" t="s">
+      <c r="G3" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="25" t="s">
+      <c r="I3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="47">
         <f>Price</f>
         <v>45</v>
       </c>
-      <c r="K3" s="43"/>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="8" t="s">
         <v>5</v>
       </c>
       <c r="B4" t="str">
         <f>Inputs!D5</f>
         <v>NIMB</v>
       </c>
-      <c r="E4" s="25" t="s">
+      <c r="E4" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="41">
+      <c r="F4" s="46">
         <f>Inputs!D10</f>
         <v>46231</v>
       </c>
-      <c r="G4" s="41"/>
-      <c r="I4" s="25" t="s">
+      <c r="I4" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="44">
         <f>Shares</f>
         <v>100</v>
       </c>
-      <c r="K4" s="38"/>
     </row>
     <row r="6">
-      <c r="B6" s="26" t="s">
+      <c r="B6" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="26"/>
-      <c r="D6" s="26"/>
-      <c r="F6" s="26" t="s">
+      <c r="C6" s="32"/>
+      <c r="D6" s="32"/>
+      <c r="F6" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="26"/>
-      <c r="H6" s="26"/>
-      <c r="J6" s="26" t="s">
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="J6" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="K6" s="26"/>
-      <c r="L6" s="26"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="32"/>
     </row>
     <row r="7">
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="40">
+      <c r="C7" s="33">
         <f>RevMy</f>
         <v>1160</v>
       </c>
-      <c r="D7" s="11"/>
-      <c r="F7" s="27" t="s">
+      <c r="D7" s="19"/>
+      <c r="F7" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="40">
+      <c r="G7" s="33">
         <f>EbitdaMy</f>
         <v>301.6</v>
       </c>
-      <c r="H7" s="11"/>
-      <c r="J7" s="27" t="s">
+      <c r="H7" s="19"/>
+      <c r="J7" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="K7" s="40">
+      <c r="K7" s="33">
         <f>NiMy</f>
         <v>156.60000000000002</v>
       </c>
-      <c r="L7" s="11"/>
+      <c r="L7" s="19"/>
     </row>
     <row r="8">
-      <c r="B8" s="27" t="s">
+      <c r="B8" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="40">
+      <c r="C8" s="33">
         <f>ConsRev</f>
         <v>1150</v>
       </c>
-      <c r="D8" s="11"/>
-      <c r="F8" s="27" t="s">
+      <c r="D8" s="19"/>
+      <c r="F8" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="40">
+      <c r="G8" s="33">
         <f>ConsEBITDA</f>
         <v>295</v>
       </c>
-      <c r="H8" s="11"/>
-      <c r="J8" s="27" t="s">
+      <c r="H8" s="19"/>
+      <c r="J8" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="K8" s="40">
+      <c r="K8" s="33">
         <f>ConsNI</f>
         <v>150</v>
       </c>
-      <c r="L8" s="11"/>
+      <c r="L8" s="19"/>
     </row>
     <row r="9">
-      <c r="B9" s="27" t="s">
+      <c r="B9" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="37">
+      <c r="C9" s="41">
         <f>RevMy/PriorRev-1</f>
         <v>0.15999999999999992</v>
       </c>
-      <c r="D9" s="11"/>
-      <c r="F9" s="27" t="s">
+      <c r="D9" s="19"/>
+      <c r="F9" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="37">
+      <c r="G9" s="41">
         <f>EbitdaMy/PriorEBITDA-1</f>
         <v>0.20640000000000014</v>
       </c>
-      <c r="H9" s="11"/>
-      <c r="J9" s="27" t="s">
+      <c r="H9" s="19"/>
+      <c r="J9" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="K9" s="37">
+      <c r="K9" s="41">
         <f>NiMy/PriorNI-1</f>
         <v>0.30500000000000016</v>
       </c>
-      <c r="L9" s="11"/>
+      <c r="L9" s="19"/>
     </row>
     <row r="10">
-      <c r="B10" s="27" t="s">
+      <c r="B10" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="37">
+      <c r="C10" s="41">
         <f>RevMy/ConsRev-1</f>
         <v>0.008695652173912993</v>
       </c>
-      <c r="D10" s="11"/>
-      <c r="F10" s="27" t="s">
+      <c r="D10" s="19"/>
+      <c r="F10" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="37">
+      <c r="G10" s="41">
         <f>EbitdaMy/ConsEBITDA-1</f>
         <v>0.022372881355932295</v>
       </c>
-      <c r="H10" s="11"/>
-      <c r="J10" s="27" t="s">
+      <c r="H10" s="19"/>
+      <c r="J10" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="K10" s="37">
+      <c r="K10" s="41">
         <f>NiMy/ConsNI-1</f>
         <v>0.04400000000000026</v>
       </c>
-      <c r="L10" s="11"/>
+      <c r="L10" s="19"/>
     </row>
     <row r="11">
-      <c r="B11" s="27" t="s">
+      <c r="B11" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="42" t="str">
+      <c r="C11" s="38" t="str">
         <f>IF(RevMy/ConsRev-1&gt;=BeatThresh,"BEAT",IF(RevMy/ConsRev-1&lt;=MissThresh,"MISS","IN-LINE"))</f>
         <v>IN-LINE</v>
       </c>
-      <c r="D11" s="11"/>
-      <c r="F11" s="27" t="s">
+      <c r="D11" s="19"/>
+      <c r="F11" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="G11" s="42" t="str">
+      <c r="G11" s="38" t="str">
         <f>IF(EbitdaMy/ConsEBITDA-1&gt;=BeatThresh,"BEAT",IF(EbitdaMy/ConsEBITDA-1&lt;=MissThresh,"MISS","IN-LINE"))</f>
         <v>BEAT</v>
       </c>
-      <c r="H11" s="11"/>
-      <c r="J11" s="27" t="s">
+      <c r="H11" s="19"/>
+      <c r="J11" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="K11" s="42" t="str">
+      <c r="K11" s="38" t="str">
         <f>IF(NiMy/ConsNI-1&gt;=BeatThresh,"BEAT",IF(NiMy/ConsNI-1&lt;=MissThresh,"MISS","IN-LINE"))</f>
         <v>BEAT</v>
       </c>
-      <c r="L11" s="11"/>
+      <c r="L11" s="19"/>
     </row>
     <row r="13">
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
-      <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
-      <c r="L13" s="7"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="11"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="11"/>
     </row>
     <row r="14">
-      <c r="B14" s="32" t="str">
+      <c r="B14" s="39" t="str">
         <f>INDEX(KpiNames,1,MATCH(SelectedSector,SectorList,0))</f>
         <v>ARR ($M)</v>
       </c>
-      <c r="C14" s="32"/>
-      <c r="D14" s="32" t="str">
+      <c r="C14" s="39"/>
+      <c r="D14" s="39" t="str">
         <f>INDEX(KpiNames,2,MATCH(SelectedSector,SectorList,0))</f>
         <v>Net Rev Retention (%)</v>
       </c>
-      <c r="E14" s="32"/>
-      <c r="F14" s="32" t="str">
+      <c r="E14" s="39"/>
+      <c r="F14" s="39" t="str">
         <f>INDEX(KpiNames,3,MATCH(SelectedSector,SectorList,0))</f>
         <v>Rule of 40 (%)</v>
       </c>
-      <c r="G14" s="32"/>
-      <c r="H14" s="32" t="str">
+      <c r="G14" s="39"/>
+      <c r="H14" s="39" t="str">
         <f>INDEX(KpiNames,4,MATCH(SelectedSector,SectorList,0))</f>
         <v>Gross Margin (%)</v>
       </c>
-      <c r="I14" s="32"/>
-      <c r="J14" s="32" t="str">
+      <c r="I14" s="39"/>
+      <c r="J14" s="39" t="str">
         <f>INDEX(KpiNames,5,MATCH(SelectedSector,SectorList,0))</f>
         <v>CAC Payback (mo)</v>
       </c>
-      <c r="K14" s="32"/>
+      <c r="K14" s="39"/>
     </row>
     <row r="15">
-      <c r="B15" s="34">
+      <c r="B15" s="36">
         <f>INDEX(KpiValues,1,MATCH(SelectedSector,SectorList,0))</f>
         <v>1200</v>
       </c>
-      <c r="C15" s="34"/>
-      <c r="D15" s="34">
+      <c r="C15" s="36"/>
+      <c r="D15" s="36">
         <f>INDEX(KpiValues,2,MATCH(SelectedSector,SectorList,0))</f>
         <v>118</v>
       </c>
-      <c r="E15" s="34"/>
-      <c r="F15" s="34">
+      <c r="E15" s="36"/>
+      <c r="F15" s="36">
         <f>INDEX(KpiValues,3,MATCH(SelectedSector,SectorList,0))</f>
         <v>46</v>
       </c>
-      <c r="G15" s="34"/>
-      <c r="H15" s="34">
+      <c r="G15" s="36"/>
+      <c r="H15" s="36">
         <f>INDEX(KpiValues,4,MATCH(SelectedSector,SectorList,0))</f>
         <v>78</v>
       </c>
-      <c r="I15" s="34"/>
-      <c r="J15" s="34">
+      <c r="I15" s="36"/>
+      <c r="J15" s="36">
         <f>INDEX(KpiValues,5,MATCH(SelectedSector,SectorList,0))</f>
         <v>14</v>
       </c>
-      <c r="K15" s="34"/>
+      <c r="K15" s="36"/>
     </row>
     <row r="17">
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
-      <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
-      <c r="L17" s="7"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="11"/>
     </row>
     <row r="18">
-      <c r="B18" s="28" t="s">
+      <c r="B18" s="37" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="D18" s="28" t="s">
+      <c r="D18" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="E18" s="28" t="s">
+      <c r="E18" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="F18" s="28" t="s">
+      <c r="F18" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="G18" s="28" t="s">
+      <c r="G18" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="H18" s="28" t="s">
+      <c r="H18" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="I18" s="28" t="s">
+      <c r="I18" s="37" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="36">
+      <c r="B19" s="35">
         <f>Valuation!C5</f>
         <v>14.423076923076922</v>
       </c>
-      <c r="C19" s="36">
+      <c r="C19" s="35">
         <f>Valuation!C6</f>
         <v>28.73563218390804</v>
       </c>
-      <c r="D19" s="36">
+      <c r="D19" s="35">
         <f>Valuation!C7</f>
         <v>3.75</v>
       </c>
-      <c r="E19" s="36">
+      <c r="E19" s="35">
         <f>Valuation!C8</f>
         <v>3.8793103448275863</v>
       </c>
-      <c r="F19" s="39">
+      <c r="F19" s="45">
         <f>FairValue</f>
         <v>45.85775303860559</v>
       </c>
-      <c r="G19" s="39">
+      <c r="G19" s="45">
         <f>AvgImplied</f>
         <v>48.165</v>
       </c>
-      <c r="H19" s="39">
+      <c r="H19" s="45">
         <f>Price</f>
         <v>45</v>
       </c>
-      <c r="I19" s="29">
+      <c r="I19" s="42">
         <f>Valuation!C35</f>
         <v>0.0190611786356798</v>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="7"/>
-      <c r="J21" s="7"/>
-      <c r="K21" s="7"/>
-      <c r="L21" s="7"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11"/>
+      <c r="I21" s="11"/>
+      <c r="J21" s="11"/>
+      <c r="K21" s="11"/>
+      <c r="L21" s="11"/>
     </row>
     <row r="22">
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D22" s="33">
+      <c r="D22" s="31">
         <f>AVERAGE(RevMy/ConsRev-1,EbitdaMy/ConsEBITDA-1,NiMy/ConsNI-1)</f>
         <v>0.025022844509948516</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="F22" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H22" s="45" t="str">
+      <c r="H22" s="40" t="str">
         <f>IF(D22&gt;=BeatThresh,"LIKELY BEAT  ▲",IF(D22&lt;=MissThresh,"LIKELY MISS  ▼","IN-LINE  ►"))</f>
         <v>LIKELY BEAT  ▲</v>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D23" s="33">
+      <c r="D23" s="31">
         <f>D22*ReactSens</f>
         <v>0.20018275607958813</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="F23" s="5" t="s">
         <v>28</v>
       </c>
       <c r="H23" t="str">
@@ -1830,97 +1828,97 @@
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="19" t="s">
+      <c r="B40" s="24" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="35" t="s">
+      <c r="B43" s="43" t="s">
         <v>30</v>
       </c>
-      <c r="C43" s="35" t="s">
+      <c r="C43" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="D43" s="35" t="s">
+      <c r="D43" s="43" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="3" t="s">
+      <c r="B44" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C44" s="1">
+      <c r="C44" s="2">
         <f>ConsRev</f>
         <v>1150</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44" s="2">
         <f>RevMy</f>
         <v>1160</v>
       </c>
     </row>
     <row r="45">
-      <c r="B45" s="3" t="s">
+      <c r="B45" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C45" s="1">
+      <c r="C45" s="2">
         <f>ConsEBITDA</f>
         <v>295</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="2">
         <f>EbitdaMy</f>
         <v>301.6</v>
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="3" t="s">
+      <c r="B46" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C46" s="1">
+      <c r="C46" s="2">
         <f>ConsNI</f>
         <v>150</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46" s="2">
         <f>NiMy</f>
         <v>156.60000000000002</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="35">
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="B17:L17"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="J6:L6"/>
     <mergeCell ref="D14:E14"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B21:L21"/>
-    <mergeCell ref="K8:L8"/>
-    <mergeCell ref="B17:L17"/>
     <mergeCell ref="H22:L22"/>
     <mergeCell ref="C9:D9"/>
-    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="B21:L21"/>
+    <mergeCell ref="H23:L23"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="G7:H7"/>
     <mergeCell ref="B40:L40"/>
-    <mergeCell ref="H23:L23"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="G11:H11"/>
     <mergeCell ref="K11:L11"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="K9:L9"/>
-    <mergeCell ref="F6:H6"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="B13:L13"/>
     <mergeCell ref="C10:D10"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B13:L13"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="K10:L10"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="B14:C14"/>
   </mergeCells>
   <conditionalFormatting sqref="H22">
     <cfRule type="expression" dxfId="0" priority="1">
@@ -2053,80 +2051,80 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
     </row>
     <row r="3">
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="F3" s="7" t="s">
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="F3" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
     </row>
     <row r="4">
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="24" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="19" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="20">
         <v>45</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="I6" s="10" t="s">
+      <c r="I6" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="J6" s="10" t="s">
+      <c r="J6" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="K6" s="10" t="s">
+      <c r="K6" s="12" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="D7" s="23">
+      <c r="D7" s="26">
         <v>100</v>
       </c>
       <c r="F7" t="s">
@@ -2138,21 +2136,21 @@
       <c r="H7" t="s">
         <v>3</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="6">
         <v>45</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="21">
         <v>100</v>
       </c>
-      <c r="K7">
+      <c r="K7" s="2">
         <v>-150</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="D8" s="17">
+      <c r="D8" s="22">
         <v>-150</v>
       </c>
       <c r="F8" t="s">
@@ -2164,21 +2162,21 @@
       <c r="H8" t="s">
         <v>49</v>
       </c>
-      <c r="I8">
+      <c r="I8" s="6">
         <v>62</v>
       </c>
-      <c r="J8">
+      <c r="J8" s="21">
         <v>210</v>
       </c>
-      <c r="K8">
+      <c r="K8" s="2">
         <v>480</v>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="18">
         <v>0.21</v>
       </c>
       <c r="F9" t="s">
@@ -2190,271 +2188,271 @@
       <c r="H9" t="s">
         <v>53</v>
       </c>
-      <c r="I9">
+      <c r="I9" s="6">
         <v>95</v>
       </c>
-      <c r="J9">
+      <c r="J9" s="21">
         <v>400</v>
       </c>
-      <c r="K9">
+      <c r="K9" s="2">
         <v>6000</v>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="23">
         <v>46231</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="D11" s="11" t="str">
+      <c r="D11" s="19" t="str">
         <f>SelectedSector</f>
         <v>Tech/SaaS</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
     </row>
     <row r="14">
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="18">
         <v>0.16</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D15" s="9">
+      <c r="D15" s="18">
         <v>0.03</v>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="D16" s="9">
+      <c r="D16" s="18">
         <v>0.26</v>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="D17" s="9">
+      <c r="D17" s="18">
         <v>0.135</v>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="18">
         <v>0.85</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="D19" s="11" t="s">
+      <c r="D19" s="19" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="17">
         <f>IF(ScenarioName="Bull",1.25,IF(ScenarioName="Bear",0.7,1))</f>
         <v>1</v>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
     </row>
     <row r="23">
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="D23" s="8">
+      <c r="D23" s="17">
         <v>13</v>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="D24" s="8">
+      <c r="D24" s="17">
         <v>22</v>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="D25" s="8">
+      <c r="D25" s="17">
         <v>5</v>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="17">
         <v>5</v>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="11"/>
     </row>
     <row r="29">
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="D29" s="9">
+      <c r="D29" s="18">
         <v>0.042</v>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="D30" s="9">
+      <c r="D30" s="18">
         <v>0.05</v>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="D31" s="21">
+      <c r="D31" s="25">
         <v>1.2</v>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="D32" s="9">
+      <c r="D32" s="18">
         <v>0.06</v>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="D33" s="9">
+      <c r="D33" s="18">
         <v>0.85</v>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="D34" s="9">
+      <c r="D34" s="18">
         <v>0.15</v>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="D35" s="9">
+      <c r="D35" s="18">
         <v>0.03</v>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="7" t="s">
+      <c r="B37" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
+      <c r="C37" s="11"/>
+      <c r="D37" s="11"/>
     </row>
     <row r="38">
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="D38" s="9">
+      <c r="D38" s="18">
         <v>0.02</v>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="D39" s="9">
+      <c r="D39" s="18">
         <v>-0.02</v>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="D40" s="8">
+      <c r="D40" s="17">
         <v>8</v>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="7" t="s">
+      <c r="B42" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="C42" s="7"/>
-      <c r="D42" s="7"/>
+      <c r="C42" s="11"/>
+      <c r="D42" s="11"/>
     </row>
     <row r="43">
-      <c r="B43" s="6" t="s">
+      <c r="B43" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="D43" s="12"/>
+      <c r="D43" s="20"/>
     </row>
     <row r="44">
-      <c r="B44" s="6" t="s">
+      <c r="B44" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="D44" s="17"/>
+      <c r="D44" s="22"/>
     </row>
     <row r="45">
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="D45" s="12"/>
+      <c r="D45" s="20"/>
     </row>
     <row r="46">
-      <c r="B46" s="6" t="s">
+      <c r="B46" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="D46" s="11"/>
+      <c r="D46" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="F3:K3"/>
+    <mergeCell ref="B37:D37"/>
     <mergeCell ref="B28:D28"/>
-    <mergeCell ref="F3:K3"/>
     <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="B13:D13"/>
     <mergeCell ref="B42:D42"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D19">
@@ -2475,83 +2473,83 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
     </row>
     <row r="3">
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="3" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="2">
         <v>1000</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>1150</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>1300</v>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="2">
         <v>250</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="2">
         <v>295</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>340</v>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="2">
         <v>120</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="2">
         <v>150</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>175</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="6">
         <f>C6/Shares</f>
         <v>1.2</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="6">
         <f>D6/Shares</f>
         <v>1.5</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="6">
         <f>E6/Shares</f>
         <v>1.75</v>
       </c>
@@ -2575,81 +2573,81 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
     </row>
     <row r="3">
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="2">
         <f>PriorRev*(1+RevGrowthMy*ScenarioMult)</f>
         <v>1160</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="24" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="2">
         <f>RevMy*EbitdaMarginMy</f>
         <v>301.6</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="24" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="2">
         <f>RevMy*NiMarginMy</f>
         <v>156.60000000000002</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="24" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="6">
         <f>NiMy/Shares</f>
         <v>1.5660000000000003</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="24" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="2">
         <f>EbitdaMy*(1-TaxRate)*FcfConv</f>
         <v>202.5244</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="24" t="s">
         <v>101</v>
       </c>
     </row>
@@ -2671,28 +2669,28 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
     </row>
     <row r="3">
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="7"/>
+      <c r="C3" s="11"/>
     </row>
     <row r="4">
       <c r="B4" t="s">
         <v>104</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="2">
         <f>Price*Shares+NetDebt</f>
         <v>4350</v>
       </c>
@@ -2701,7 +2699,7 @@
       <c r="B5" t="s">
         <v>105</v>
       </c>
-      <c r="C5" s="15">
+      <c r="C5" s="14">
         <f>EV/EbitdaMy</f>
         <v>14.423076923076922</v>
       </c>
@@ -2710,7 +2708,7 @@
       <c r="B6" t="s">
         <v>106</v>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="14">
         <f>Price/EpsMy</f>
         <v>28.73563218390804</v>
       </c>
@@ -2719,7 +2717,7 @@
       <c r="B7" t="s">
         <v>107</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="14">
         <f>EV/RevMy</f>
         <v>3.75</v>
       </c>
@@ -2728,22 +2726,22 @@
       <c r="B8" t="s">
         <v>108</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="14">
         <f>Price*Shares/RevMy</f>
         <v>3.8793103448275863</v>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="C10" s="7"/>
+      <c r="C10" s="11"/>
     </row>
     <row r="11">
       <c r="B11" t="s">
         <v>110</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="6">
         <f>(PeerEVEBITDA*EbitdaMy-NetDebt)/Shares</f>
         <v>40.708</v>
       </c>
@@ -2752,7 +2750,7 @@
       <c r="B12" t="s">
         <v>111</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="6">
         <f>PeerPE*EpsMy</f>
         <v>34.452000000000005</v>
       </c>
@@ -2761,7 +2759,7 @@
       <c r="B13" t="s">
         <v>112</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="6">
         <f>(PeerEVRev*RevMy-NetDebt)/Shares</f>
         <v>59.5</v>
       </c>
@@ -2770,31 +2768,31 @@
       <c r="B14" t="s">
         <v>113</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C14" s="6">
         <f>PeerPS*RevMy/Shares</f>
         <v>58</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="C15" s="24">
+      <c r="C15" s="28">
         <f>AVERAGE(C11:C14)</f>
         <v>48.165</v>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="C17" s="7"/>
+      <c r="C17" s="11"/>
     </row>
     <row r="18">
       <c r="B18" t="s">
         <v>116</v>
       </c>
-      <c r="C18" s="13">
+      <c r="C18" s="10">
         <f>RiskFree+Beta*ERP</f>
         <v>0.10200000000000001</v>
       </c>
@@ -2803,147 +2801,147 @@
       <c r="B19" t="s">
         <v>117</v>
       </c>
-      <c r="C19" s="13">
+      <c r="C19" s="10">
         <f>CostDebt*(1-TaxRate)</f>
         <v>0.0474</v>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="C20" s="16">
+      <c r="C20" s="15">
         <f>WeightEquity*C18+WeightDebt*C19</f>
         <v>0.09381</v>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="7"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="11"/>
     </row>
     <row r="23">
-      <c r="B23" s="20" t="s">
+      <c r="B23" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="C23" s="20">
+      <c r="C23" s="9">
         <v>1</v>
       </c>
-      <c r="D23" s="20">
+      <c r="D23" s="9">
         <v>2</v>
       </c>
-      <c r="E23" s="20">
+      <c r="E23" s="9">
         <v>3</v>
       </c>
-      <c r="F23" s="20">
+      <c r="F23" s="9">
         <v>4</v>
       </c>
-      <c r="G23" s="20">
+      <c r="G23" s="9">
         <v>5</v>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="C24" s="13">
+      <c r="C24" s="10">
         <f>MAX(RevGrowthMy*ScenarioMult,TermGrowth)</f>
         <v>0.16</v>
       </c>
-      <c r="D24" s="13">
+      <c r="D24" s="10">
         <f>MAX(C24-GrowthFade,TermGrowth)</f>
         <v>0.13</v>
       </c>
-      <c r="E24" s="13">
+      <c r="E24" s="10">
         <f>MAX(D24-GrowthFade,TermGrowth)</f>
         <v>0.1</v>
       </c>
-      <c r="F24" s="13">
+      <c r="F24" s="10">
         <f>MAX(E24-GrowthFade,TermGrowth)</f>
         <v>0.07</v>
       </c>
-      <c r="G24" s="13">
+      <c r="G24" s="10">
         <f>MAX(F24-GrowthFade,TermGrowth)</f>
         <v>0.04000000000000001</v>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="C25" s="1">
+      <c r="C25" s="2">
         <f>RevMy*(1+C24)</f>
         <v>1345.6</v>
       </c>
-      <c r="D25" s="1">
+      <c r="D25" s="2">
         <f>C25*(1+D24)</f>
         <v>1520.5279999999998</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <f>D25*(1+E24)</f>
         <v>1672.5808</v>
       </c>
-      <c r="F25" s="1">
+      <c r="F25" s="2">
         <f>E25*(1+F24)</f>
         <v>1789.661456</v>
       </c>
-      <c r="G25" s="1">
+      <c r="G25" s="2">
         <f>F25*(1+G24)</f>
         <v>1861.24791424</v>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C26" s="1">
+      <c r="C26" s="2">
         <f>C25*EbitdaMarginMy</f>
         <v>349.856</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="2">
         <f>D25*EbitdaMarginMy</f>
         <v>395.33727999999996</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <f>E25*EbitdaMarginMy</f>
         <v>434.871008</v>
       </c>
-      <c r="F26" s="1">
+      <c r="F26" s="2">
         <f>F25*EbitdaMarginMy</f>
         <v>465.31197856</v>
       </c>
-      <c r="G26" s="1">
+      <c r="G26" s="2">
         <f>G25*EbitdaMarginMy</f>
         <v>483.9244577024</v>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="C27" s="1">
+      <c r="C27" s="2">
         <f>C26*(1-TaxRate)*FcfConv</f>
         <v>234.92830399999997</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27" s="2">
         <f>D26*(1-TaxRate)*FcfConv</f>
         <v>265.46898351999994</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <f>E26*(1-TaxRate)*FcfConv</f>
         <v>292.015881872</v>
       </c>
-      <c r="F27" s="1">
+      <c r="F27" s="2">
         <f>F26*(1-TaxRate)*FcfConv</f>
         <v>312.45699360304</v>
       </c>
-      <c r="G27" s="1">
+      <c r="G27" s="2">
         <f>G26*(1-TaxRate)*FcfConv</f>
         <v>324.95527334716155</v>
       </c>
@@ -2952,7 +2950,7 @@
       <c r="B29" t="s">
         <v>123</v>
       </c>
-      <c r="C29" s="1">
+      <c r="C29" s="2">
         <f>NPV(WACC,C27:G27)</f>
         <v>1085.6378864760316</v>
       </c>
@@ -2961,7 +2959,7 @@
       <c r="B30" t="s">
         <v>124</v>
       </c>
-      <c r="C30" s="1">
+      <c r="C30" s="2">
         <f>G27*(1+TermGrowth)/(WACC-TermGrowth)</f>
         <v>5245.320977081592</v>
       </c>
@@ -2970,34 +2968,34 @@
       <c r="B31" t="s">
         <v>125</v>
       </c>
-      <c r="C31" s="1">
+      <c r="C31" s="2">
         <f>C30/(1+WACC)^5</f>
         <v>3350.137417384527</v>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="C32" s="1">
+      <c r="C32" s="2">
         <f>C29+C31</f>
         <v>4435.775303860559</v>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="C33" s="1">
+      <c r="C33" s="2">
         <f>C32-NetDebt</f>
         <v>4585.775303860559</v>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="C34" s="22">
+      <c r="C34" s="27">
         <f>C33/Shares</f>
         <v>45.85775303860559</v>
       </c>
@@ -3006,185 +3004,185 @@
       <c r="B35" t="s">
         <v>129</v>
       </c>
-      <c r="C35" s="30">
+      <c r="C35" s="29">
         <f>FairValue/Price-1</f>
         <v>0.0190611786356798</v>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="7" t="s">
+      <c r="B37" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
-      <c r="E37" s="7"/>
-      <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
-      <c r="H37" s="7"/>
+      <c r="C37" s="11"/>
+      <c r="D37" s="11"/>
+      <c r="E37" s="11"/>
+      <c r="F37" s="11"/>
+      <c r="G37" s="11"/>
+      <c r="H37" s="11"/>
     </row>
     <row r="38">
-      <c r="B38" s="31" t="s">
+      <c r="B38" s="30" t="s">
         <v>131</v>
       </c>
-      <c r="C38" s="31">
+      <c r="C38" s="30">
         <f>TermGrowth+-0.01</f>
         <v>0.019999999999999997</v>
       </c>
-      <c r="D38" s="31">
+      <c r="D38" s="30">
         <f>TermGrowth+-0.005</f>
         <v>0.024999999999999998</v>
       </c>
-      <c r="E38" s="31">
+      <c r="E38" s="30">
         <f>TermGrowth+0</f>
         <v>0.03</v>
       </c>
-      <c r="F38" s="31">
+      <c r="F38" s="30">
         <f>TermGrowth+0.005</f>
         <v>0.034999999999999996</v>
       </c>
-      <c r="G38" s="31">
+      <c r="G38" s="30">
         <f>TermGrowth+0.01</f>
         <v>0.04</v>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="16">
+      <c r="B39" s="15">
         <f>WACC+-0.01</f>
         <v>0.08381000000000001</v>
       </c>
-      <c r="C39" s="14">
+      <c r="C39" s="13">
         <f>(NPV($B39,$C$27:$G$27)+($G$27*(1+C$38)/($B39-C$38))/(1+$B39)^5-NetDebt)/Shares</f>
         <v>47.39403874756321</v>
       </c>
-      <c r="D39" s="14">
+      <c r="D39" s="13">
         <f>(NPV($B39,$C$27:$G$27)+($G$27*(1+D$38)/($B39-D$38))/(1+$B39)^5-NetDebt)/Shares</f>
         <v>50.53195287280684</v>
       </c>
-      <c r="E39" s="14">
+      <c r="E39" s="13">
         <f>(NPV($B39,$C$27:$G$27)+($G$27*(1+E$38)/($B39-E$38))/(1+$B39)^5-NetDebt)/Shares</f>
         <v>54.253014020024786</v>
       </c>
-      <c r="F39" s="14">
+      <c r="F39" s="13">
         <f>(NPV($B39,$C$27:$G$27)+($G$27*(1+F$38)/($B39-F$38))/(1+$B39)^5-NetDebt)/Shares</f>
         <v>58.73643147685507</v>
       </c>
-      <c r="G39" s="14">
+      <c r="G39" s="13">
         <f>(NPV($B39,$C$27:$G$27)+($G$27*(1+G$38)/($B39-G$38))/(1+$B39)^5-NetDebt)/Shares</f>
         <v>64.24322657733528</v>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="16">
+      <c r="B40" s="15">
         <f>WACC+-0.005</f>
         <v>0.08881</v>
       </c>
-      <c r="C40" s="14">
+      <c r="C40" s="13">
         <f>(NPV($B40,$C$27:$G$27)+($G$27*(1+C$38)/($B40-C$38))/(1+$B40)^5-NetDebt)/Shares</f>
         <v>43.98434802278164</v>
       </c>
-      <c r="D40" s="14">
+      <c r="D40" s="13">
         <f>(NPV($B40,$C$27:$G$27)+($G$27*(1+D$38)/($B40-D$38))/(1+$B40)^5-NetDebt)/Shares</f>
         <v>46.61731181734158</v>
       </c>
-      <c r="E40" s="14">
+      <c r="E40" s="13">
         <f>(NPV($B40,$C$27:$G$27)+($G$27*(1+E$38)/($B40-E$38))/(1+$B40)^5-NetDebt)/Shares</f>
         <v>49.69798242954478</v>
       </c>
-      <c r="F40" s="14">
+      <c r="F40" s="13">
         <f>(NPV($B40,$C$27:$G$27)+($G$27*(1+F$38)/($B40-F$38))/(1+$B40)^5-NetDebt)/Shares</f>
         <v>53.35116198287474</v>
       </c>
-      <c r="G40" s="14">
+      <c r="G40" s="13">
         <f>(NPV($B40,$C$27:$G$27)+($G$27*(1+G$38)/($B40-G$38))/(1+$B40)^5-NetDebt)/Shares</f>
         <v>57.75279053299431</v>
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="16">
+      <c r="B41" s="15">
         <f>WACC+0</f>
         <v>0.09381</v>
       </c>
-      <c r="C41" s="14">
+      <c r="C41" s="13">
         <f>(NPV($B41,$C$27:$G$27)+($G$27*(1+C$38)/($B41-C$38))/(1+$B41)^5-NetDebt)/Shares</f>
         <v>41.03769707161954</v>
       </c>
-      <c r="D41" s="14">
+      <c r="D41" s="13">
         <f>(NPV($B41,$C$27:$G$27)+($G$27*(1+D$38)/($B41-D$38))/(1+$B41)^5-NetDebt)/Shares</f>
         <v>43.27260312635998</v>
       </c>
-      <c r="E41" s="14">
+      <c r="E41" s="13">
         <f>(NPV($B41,$C$27:$G$27)+($G$27*(1+E$38)/($B41-E$38))/(1+$B41)^5-NetDebt)/Shares</f>
         <v>45.85775303860559</v>
       </c>
-      <c r="F41" s="14">
+      <c r="F41" s="13">
         <f>(NPV($B41,$C$27:$G$27)+($G$27*(1+F$38)/($B41-F$38))/(1+$B41)^5-NetDebt)/Shares</f>
         <v>48.882479538548104</v>
       </c>
-      <c r="G41" s="14">
+      <c r="G41" s="13">
         <f>(NPV($B41,$C$27:$G$27)+($G$27*(1+G$38)/($B41-G$38))/(1+$B41)^5-NetDebt)/Shares</f>
         <v>52.469318378193755</v>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="16">
+      <c r="B42" s="15">
         <f>WACC+0.005</f>
         <v>0.09881000000000001</v>
       </c>
-      <c r="C42" s="14">
+      <c r="C42" s="13">
         <f>(NPV($B42,$C$27:$G$27)+($G$27*(1+C$38)/($B42-C$38))/(1+$B42)^5-NetDebt)/Shares</f>
         <v>38.465933352713236</v>
       </c>
-      <c r="D42" s="14">
+      <c r="D42" s="13">
         <f>(NPV($B42,$C$27:$G$27)+($G$27*(1+D$38)/($B42-D$38))/(1+$B42)^5-NetDebt)/Shares</f>
         <v>40.381982514036416</v>
       </c>
-      <c r="E42" s="14">
+      <c r="E42" s="13">
         <f>(NPV($B42,$C$27:$G$27)+($G$27*(1+E$38)/($B42-E$38))/(1+$B42)^5-NetDebt)/Shares</f>
         <v>42.576486719876854</v>
       </c>
-      <c r="F42" s="14">
+      <c r="F42" s="13">
         <f>(NPV($B42,$C$27:$G$27)+($G$27*(1+F$38)/($B42-F$38))/(1+$B42)^5-NetDebt)/Shares</f>
         <v>45.114903197436526</v>
       </c>
-      <c r="G42" s="14">
+      <c r="G42" s="13">
         <f>(NPV($B42,$C$27:$G$27)+($G$27*(1+G$38)/($B42-G$38))/(1+$B42)^5-NetDebt)/Shares</f>
         <v>48.08494975109885</v>
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="16">
+      <c r="B43" s="15">
         <f>WACC+0.01</f>
         <v>0.10381</v>
       </c>
-      <c r="C43" s="14">
+      <c r="C43" s="13">
         <f>(NPV($B43,$C$27:$G$27)+($G$27*(1+C$38)/($B43-C$38))/(1+$B43)^5-NetDebt)/Shares</f>
         <v>36.201941148015415</v>
       </c>
-      <c r="D43" s="14">
+      <c r="D43" s="13">
         <f>(NPV($B43,$C$27:$G$27)+($G$27*(1+D$38)/($B43-D$38))/(1+$B43)^5-NetDebt)/Shares</f>
         <v>37.85900456016365</v>
       </c>
-      <c r="E43" s="14">
+      <c r="E43" s="13">
         <f>(NPV($B43,$C$27:$G$27)+($G$27*(1+E$38)/($B43-E$38))/(1+$B43)^5-NetDebt)/Shares</f>
         <v>39.74057188941638</v>
       </c>
-      <c r="F43" s="14">
+      <c r="F43" s="13">
         <f>(NPV($B43,$C$27:$G$27)+($G$27*(1+F$38)/($B43-F$38))/(1+$B43)^5-NetDebt)/Shares</f>
         <v>41.895583097357196</v>
       </c>
-      <c r="G43" s="14">
+      <c r="G43" s="13">
         <f>(NPV($B43,$C$27:$G$27)+($G$27*(1+G$38)/($B43-G$38))/(1+$B43)^5-NetDebt)/Shares</f>
         <v>44.38831742204161</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="B37:H37"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B17:C17"/>
     <mergeCell ref="B22:H22"/>
-    <mergeCell ref="B37:H37"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B17:C17"/>
   </mergeCells>
   <conditionalFormatting sqref="C39:G43">
     <cfRule type="colorScale" priority="1">
@@ -3212,37 +3210,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
     </row>
     <row r="3">
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="3" t="s">
         <v>136</v>
       </c>
     </row>
@@ -3250,27 +3248,27 @@
       <c r="B4" t="s">
         <v>63</v>
       </c>
-      <c r="C4" s="13">
+      <c r="C4" s="10">
         <f>RevGrowthMy</f>
         <v>0.16</v>
       </c>
-      <c r="D4" s="13">
+      <c r="D4" s="10">
         <f>EbitdaMarginMy</f>
         <v>0.26</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <f>PriorRev*(1+C4)</f>
         <v>1160</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4" s="2">
         <f>E4*D4</f>
         <v>301.6</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="6">
         <f>(PeerEVEBITDA*F4-NetDebt)/Shares</f>
         <v>40.708</v>
       </c>
-      <c r="H4" s="13">
+      <c r="H4" s="10">
         <f>G4/Price-1</f>
         <v>-0.09537777777777778</v>
       </c>
@@ -3279,27 +3277,27 @@
       <c r="B5" t="s">
         <v>137</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="10">
         <f>RevGrowthMy*1.25</f>
         <v>0.2</v>
       </c>
-      <c r="D5" s="13">
+      <c r="D5" s="10">
         <f>EbitdaMarginMy+0.03</f>
         <v>0.29000000000000004</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <f>PriorRev*(1+C5)</f>
         <v>1200</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="2">
         <f>E5*D5</f>
         <v>348.00000000000006</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="6">
         <f>(PeerEVEBITDA*F5-NetDebt)/Shares</f>
         <v>46.74000000000001</v>
       </c>
-      <c r="H5" s="13">
+      <c r="H5" s="10">
         <f>G5/Price-1</f>
         <v>0.03866666666666685</v>
       </c>
@@ -3308,53 +3306,53 @@
       <c r="B6" t="s">
         <v>138</v>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="10">
         <f>RevGrowthMy*0.7</f>
         <v>0.11199999999999999</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="10">
         <f>EbitdaMarginMy-0.04</f>
         <v>0.22</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <f>PriorRev*(1+C6)</f>
         <v>1112</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="2">
         <f>E6*D6</f>
         <v>244.64000000000001</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="6">
         <f>(PeerEVEBITDA*F6-NetDebt)/Shares</f>
         <v>33.303200000000004</v>
       </c>
-      <c r="H6" s="13">
+      <c r="H6" s="10">
         <f>G6/Price-1</f>
         <v>-0.25992888888888876</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
     </row>
     <row r="9">
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="12" t="s">
         <v>143</v>
       </c>
     </row>
@@ -3362,15 +3360,15 @@
       <c r="B10" t="s">
         <v>144</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="6">
         <f>(PeerEVEBITDA*(PriorRev*(1+RevGrowthMy*0.8)*EbitdaMarginMy)-NetDebt)/Shares</f>
         <v>39.626400000000004</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="6">
         <f>(PeerEVEBITDA*(PriorRev*(1+RevGrowthMy*1.2)*EbitdaMarginMy)-NetDebt)/Shares</f>
         <v>41.7896</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="6">
         <f>ABS(D10-C10)</f>
         <v>2.1631999999999962</v>
       </c>
@@ -3379,15 +3377,15 @@
       <c r="B11" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="6">
         <f>(PeerEVEBITDA*(PriorRev*(1+RevGrowthMy)*EbitdaMarginMy*0.8)-NetDebt)/Shares</f>
         <v>32.866400000000006</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="6">
         <f>(PeerEVEBITDA*(PriorRev*(1+RevGrowthMy)*EbitdaMarginMy*1.2)-NetDebt)/Shares</f>
         <v>48.5496</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="6">
         <f>ABS(D11-C11)</f>
         <v>15.683199999999992</v>
       </c>
@@ -3396,15 +3394,15 @@
       <c r="B12" t="s">
         <v>66</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="6">
         <f>(PeerEVEBITDA*0.8*(PriorRev*(1+RevGrowthMy)*EbitdaMarginMy)-NetDebt)/Shares</f>
         <v>32.866400000000006</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="6">
         <f>(PeerEVEBITDA*1.2*(PriorRev*(1+RevGrowthMy)*EbitdaMarginMy)-NetDebt)/Shares</f>
         <v>48.5496</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="6">
         <f>ABS(D12-C12)</f>
         <v>15.683199999999992</v>
       </c>
@@ -3413,15 +3411,15 @@
       <c r="B13" t="s">
         <v>145</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="6">
         <f>(PeerEVEBITDA*(PriorRev*(1+RevGrowthMy)*EbitdaMarginMy)-NetDebt*1.2)/Shares</f>
         <v>41.008</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="6">
         <f>(PeerEVEBITDA*(PriorRev*(1+RevGrowthMy)*EbitdaMarginMy)-NetDebt*0.8)/Shares</f>
         <v>40.408</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="6">
         <f>ABS(D13-C13)</f>
         <v>0.6000000000000014</v>
       </c>
@@ -3430,23 +3428,23 @@
       <c r="B14" t="s">
         <v>146</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C14" s="6">
         <f>(PeerEVEBITDA*(PriorRev*(1+RevGrowthMy)*EbitdaMarginMy)-NetDebt)/Shares*1.2</f>
         <v>48.849599999999995</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="6">
         <f>(PeerEVEBITDA*(PriorRev*(1+RevGrowthMy)*EbitdaMarginMy)-NetDebt)/Shares*0.8</f>
         <v>32.5664</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="6">
         <f>ABS(D14-C14)</f>
         <v>16.283199999999994</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="B8:H8"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="B8:H8"/>
   </mergeCells>
   <conditionalFormatting sqref="H4:H6">
     <cfRule dxfId="0" type="cellIs" priority="1" operator="greaterThan">
@@ -3469,23 +3467,23 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>31</v>
       </c>
     </row>
@@ -3493,11 +3491,11 @@
       <c r="A4" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="2">
         <f>ConsRev</f>
         <v>1150</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="2">
         <f>RevMy</f>
         <v>1160</v>
       </c>
@@ -3506,11 +3504,11 @@
       <c r="A5" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="2">
         <f>ConsEBITDA</f>
         <v>295</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="2">
         <f>EbitdaMy</f>
         <v>301.6</v>
       </c>
@@ -3519,20 +3517,20 @@
       <c r="A6" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="2">
         <f>ConsNI</f>
         <v>150</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="2">
         <f>NiMy</f>
         <v>156.60000000000002</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>149</v>
       </c>
     </row>
@@ -3541,7 +3539,7 @@
         <f>INDEX(KpiNames,1,MATCH(SelectedSector,SectorList,0))</f>
         <v>ARR ($M)</v>
       </c>
-      <c r="B10" s="46">
+      <c r="B10" s="4">
         <f>INDEX(KpiValues,1,MATCH(SelectedSector,SectorList,0))</f>
         <v>1200</v>
       </c>
@@ -3551,7 +3549,7 @@
         <f>INDEX(KpiNames,2,MATCH(SelectedSector,SectorList,0))</f>
         <v>Net Rev Retention (%)</v>
       </c>
-      <c r="B11" s="46">
+      <c r="B11" s="4">
         <f>INDEX(KpiValues,2,MATCH(SelectedSector,SectorList,0))</f>
         <v>118</v>
       </c>
@@ -3561,7 +3559,7 @@
         <f>INDEX(KpiNames,3,MATCH(SelectedSector,SectorList,0))</f>
         <v>Rule of 40 (%)</v>
       </c>
-      <c r="B12" s="46">
+      <c r="B12" s="4">
         <f>INDEX(KpiValues,3,MATCH(SelectedSector,SectorList,0))</f>
         <v>46</v>
       </c>
@@ -3571,7 +3569,7 @@
         <f>INDEX(KpiNames,4,MATCH(SelectedSector,SectorList,0))</f>
         <v>Gross Margin (%)</v>
       </c>
-      <c r="B13" s="46">
+      <c r="B13" s="4">
         <f>INDEX(KpiValues,4,MATCH(SelectedSector,SectorList,0))</f>
         <v>78</v>
       </c>
@@ -3581,16 +3579,16 @@
         <f>INDEX(KpiNames,5,MATCH(SelectedSector,SectorList,0))</f>
         <v>CAC Payback (mo)</v>
       </c>
-      <c r="B14" s="46">
+      <c r="B14" s="4">
         <f>INDEX(KpiValues,5,MATCH(SelectedSector,SectorList,0))</f>
         <v>14</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>149</v>
       </c>
     </row>
@@ -3598,7 +3596,7 @@
       <c r="A18" t="s">
         <v>151</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B18" s="2">
         <f>ConsNI</f>
         <v>150</v>
       </c>
@@ -3607,7 +3605,7 @@
       <c r="A19" t="s">
         <v>152</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B19" s="2">
         <f>(RevMy-ConsRev)*NiMarginMy</f>
         <v>1.35</v>
       </c>
@@ -3616,7 +3614,7 @@
       <c r="A20" t="s">
         <v>153</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B20" s="2">
         <f>NiMy-ConsNI-((RevMy-ConsRev)*NiMarginMy)</f>
         <v>5.250000000000023</v>
       </c>
@@ -3625,7 +3623,7 @@
       <c r="A21" t="s">
         <v>154</v>
       </c>
-      <c r="B21" s="1">
+      <c r="B21" s="2">
         <f>NiMy</f>
         <v>156.60000000000002</v>
       </c>
@@ -3647,46 +3645,46 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
     </row>
     <row r="3">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="E3" s="20" t="s">
+      <c r="E3" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="G3" s="20" t="s">
+      <c r="G3" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="H3" s="20" t="s">
+      <c r="H3" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="I3" s="20" t="s">
+      <c r="I3" s="9" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="25"/>
+      <c r="A4" s="8"/>
       <c r="C4" t="s">
         <v>161</v>
       </c>
@@ -3710,7 +3708,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="25"/>
+      <c r="A5" s="8"/>
       <c r="C5" t="s">
         <v>168</v>
       </c>
@@ -3734,7 +3732,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="25"/>
+      <c r="A6" s="8"/>
       <c r="C6" t="s">
         <v>174</v>
       </c>
@@ -3758,7 +3756,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="25"/>
+      <c r="A7" s="8"/>
       <c r="C7" t="s">
         <v>169</v>
       </c>
@@ -3782,7 +3780,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="25"/>
+      <c r="A8" s="8"/>
       <c r="C8" t="s">
         <v>185</v>
       </c>
@@ -3806,148 +3804,148 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="8" t="s">
         <v>191</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="D10" s="20" t="s">
+      <c r="D10" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="E10" s="20" t="s">
+      <c r="E10" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="F10" s="20" t="s">
+      <c r="F10" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="H10" s="20" t="s">
+      <c r="H10" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="I10" s="20" t="s">
+      <c r="I10" s="9" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="25"/>
-      <c r="C11" s="47">
+      <c r="A11" s="8"/>
+      <c r="C11" s="7">
         <v>1200</v>
       </c>
-      <c r="D11" s="47">
+      <c r="D11" s="7">
         <v>4.5</v>
       </c>
-      <c r="E11" s="47">
+      <c r="E11" s="7">
         <v>22</v>
       </c>
-      <c r="F11" s="47">
+      <c r="F11" s="7">
         <v>1.08</v>
       </c>
-      <c r="G11" s="47">
+      <c r="G11" s="7">
         <v>3.2</v>
       </c>
-      <c r="H11" s="47">
+      <c r="H11" s="7">
         <v>520</v>
       </c>
-      <c r="I11" s="47">
+      <c r="I11" s="7">
         <v>12</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="25"/>
-      <c r="C12" s="47">
+      <c r="A12" s="8"/>
+      <c r="C12" s="7">
         <v>118</v>
       </c>
-      <c r="D12" s="47">
+      <c r="D12" s="7">
         <v>42</v>
       </c>
-      <c r="E12" s="47">
+      <c r="E12" s="7">
         <v>12</v>
       </c>
-      <c r="F12" s="47">
+      <c r="F12" s="7">
         <v>84</v>
       </c>
-      <c r="G12" s="47">
+      <c r="G12" s="7">
         <v>58</v>
       </c>
-      <c r="H12" s="47">
+      <c r="H12" s="7">
         <v>68</v>
       </c>
-      <c r="I12" s="47">
+      <c r="I12" s="7">
         <v>55</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="25"/>
-      <c r="C13" s="47">
+      <c r="A13" s="8"/>
+      <c r="C13" s="7">
         <v>46</v>
       </c>
-      <c r="D13" s="47">
+      <c r="D13" s="7">
         <v>5.2</v>
       </c>
-      <c r="E13" s="47">
+      <c r="E13" s="7">
         <v>340</v>
       </c>
-      <c r="F13" s="47">
+      <c r="F13" s="7">
         <v>2300</v>
       </c>
-      <c r="G13" s="47">
+      <c r="G13" s="7">
         <v>13.5</v>
       </c>
-      <c r="H13" s="47">
+      <c r="H13" s="7">
         <v>12.5</v>
       </c>
-      <c r="I13" s="47">
+      <c r="I13" s="7">
         <v>20</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="25"/>
-      <c r="C14" s="47">
+      <c r="A14" s="8"/>
+      <c r="C14" s="7">
         <v>78</v>
       </c>
-      <c r="D14" s="47">
+      <c r="D14" s="7">
         <v>1450</v>
       </c>
-      <c r="E14" s="47">
+      <c r="E14" s="7">
         <v>74</v>
       </c>
-      <c r="F14" s="47">
+      <c r="F14" s="7">
         <v>16</v>
       </c>
-      <c r="G14" s="47">
+      <c r="G14" s="7">
         <v>12.2</v>
       </c>
-      <c r="H14" s="47">
+      <c r="H14" s="7">
         <v>9.4</v>
       </c>
-      <c r="I14" s="47">
+      <c r="I14" s="7">
         <v>18</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="25"/>
-      <c r="C15" s="47">
+      <c r="A15" s="8"/>
+      <c r="C15" s="7">
         <v>14</v>
       </c>
-      <c r="D15" s="47">
+      <c r="D15" s="7">
         <v>31</v>
       </c>
-      <c r="E15" s="47">
+      <c r="E15" s="7">
         <v>28</v>
       </c>
-      <c r="F15" s="47">
+      <c r="F15" s="7">
         <v>13</v>
       </c>
-      <c r="G15" s="47">
+      <c r="G15" s="7">
         <v>7</v>
       </c>
-      <c r="H15" s="47">
+      <c r="H15" s="7">
         <v>11</v>
       </c>
-      <c r="I15" s="47">
+      <c r="I15" s="7">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Goldman upgrade (Stage 2): Comparable-companies tab with dynamic peer set
New Comps sheet adapted from the CRWD model's Compsheet:
- Peer set pulled from CapIQ's auto comp set (IQ_COMPARABLE_COMPANIES, indexed)
  with a curated sector-default fallback; editable in column A.
- Per-peer live pulls: company, price, market cap, EV (IQ_TEV or mktcap+net
  debt), and NTM EV/Revenue, EV/EBITDA, P/E. All IFERROR-guarded.
- Peer MEDIAN multiples -> implied value applied to our consensus EBITDA/Rev/NI
  (EV multiples run through the equity bridge), with an average implied price
  and upside vs current. CompsImplied named range exposed.
- Static presets show the default peer tickers + a 'populates in CapIQ mode'
  note (data cells blank). README updated.
</commit_message>
<xml_diff>
--- a/Sector_Consensus_vs_My_Model.xlsx
+++ b/Sector_Consensus_vs_My_Model.xlsx
@@ -13,17 +13,22 @@
     <sheet name="Scenarios" sheetId="6" r:id="rId6"/>
     <sheet name="Charts" sheetId="7" r:id="rId7"/>
     <sheet name="SectorKPIs" sheetId="8" r:id="rId8"/>
+    <sheet name="Comps" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="AnalystTgt">Valuation!$J$15</definedName>
+    <definedName name="Associates">Inputs!$D$59</definedName>
     <definedName name="AvgImplied">Valuation!$C$15</definedName>
     <definedName name="BeatThresh">Inputs!$D$38</definedName>
     <definedName name="Beta">Inputs!$D$31</definedName>
+    <definedName name="CapexPct">Inputs!$D$52</definedName>
+    <definedName name="CompsImplied">Comps!$E$20</definedName>
     <definedName name="ConsEBITDA">Consensus!$D$5</definedName>
     <definedName name="ConsEPS">Consensus!$D$7</definedName>
     <definedName name="ConsNI">Consensus!$D$6</definedName>
     <definedName name="ConsRev">Consensus!$D$4</definedName>
     <definedName name="CostDebt">Inputs!$D$32</definedName>
+    <definedName name="DaPct">Inputs!$D$53</definedName>
     <definedName name="DcfExit">Valuation!$J$13</definedName>
     <definedName name="ERP">Inputs!$D$30</definedName>
     <definedName name="EV">Valuation!$C$4</definedName>
@@ -36,10 +41,12 @@
     <definedName name="GrowthFade">Inputs!$D$15</definedName>
     <definedName name="KpiNames">SectorKPIs!$C$4:$I$8</definedName>
     <definedName name="KpiValues">SectorKPIs!$C$11:$I$15</definedName>
+    <definedName name="Minorities">Inputs!$D$58</definedName>
     <definedName name="MissThresh">Inputs!$D$39</definedName>
     <definedName name="NetDebt">Inputs!$D$8</definedName>
     <definedName name="NiMarginMy">Inputs!$D$17</definedName>
     <definedName name="NiMy">MyModel!$C$6</definedName>
+    <definedName name="NwcPct">Inputs!$D$54</definedName>
     <definedName name="PeerEVEBITDA">Inputs!$D$23</definedName>
     <definedName name="PeerEVRev">Inputs!$D$25</definedName>
     <definedName name="PeerPE">Inputs!$D$24</definedName>
@@ -52,6 +59,8 @@
     <definedName name="RevGrowthMy">Inputs!$D$14</definedName>
     <definedName name="RevMy">MyModel!$C$4</definedName>
     <definedName name="RiskFree">Inputs!$D$29</definedName>
+    <definedName name="SbcDeduct">Inputs!$D$57</definedName>
+    <definedName name="SbcPct">Inputs!$D$55</definedName>
     <definedName name="ScenarioMult">Inputs!$D$20</definedName>
     <definedName name="ScenarioName">Inputs!$D$19</definedName>
     <definedName name="SectorList">SectorKPIs!$C$3:$I$3</definedName>
@@ -59,6 +68,7 @@
     <definedName name="Shares">Inputs!$D$7</definedName>
     <definedName name="TaxRate">Inputs!$D$9</definedName>
     <definedName name="TermGrowth">Inputs!$D$35</definedName>
+    <definedName name="TermMargin">Inputs!$D$56</definedName>
     <definedName name="Ticker">Inputs!$D$5</definedName>
     <definedName name="ValMid">Valuation!$J$21</definedName>
     <definedName name="WACC">Valuation!$C$20</definedName>
@@ -70,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="248">
   <si>
     <t>SECTOR CONSENSUS  vs  MY MODEL  —  EQUITY DASHBOARD</t>
   </si>
@@ -339,6 +349,33 @@
     <t>Last Updated</t>
   </si>
   <si>
+    <t>ADVANCED DCF / FCF</t>
+  </si>
+  <si>
+    <t>Capex (% of revenue)</t>
+  </si>
+  <si>
+    <t>D&amp;A (% of revenue)</t>
+  </si>
+  <si>
+    <t>Change in NWC (% of ΔRevenue)</t>
+  </si>
+  <si>
+    <t>Stock-based comp (% of revenue)</t>
+  </si>
+  <si>
+    <t>Terminal EBITDA Margin</t>
+  </si>
+  <si>
+    <t>Deduct SBC in FCF? (1=post-SBC, 0=pre-SBC)</t>
+  </si>
+  <si>
+    <t>Minority Interest ($M)</t>
+  </si>
+  <si>
+    <t>Associates / Investments ($M)</t>
+  </si>
+  <si>
     <t>MARKET CONSENSUS</t>
   </si>
   <si>
@@ -501,10 +538,19 @@
     <t>Revenue ($M)</t>
   </si>
   <si>
-    <t>FCF ($M)</t>
-  </si>
-  <si>
-    <t>PV of explicit FCF</t>
+    <t>FORWARD MULTIPLES (on consensus)</t>
+  </si>
+  <si>
+    <t>Unlevered FCF ($M)</t>
+  </si>
+  <si>
+    <t>Current FY</t>
+  </si>
+  <si>
+    <t>NTM</t>
+  </si>
+  <si>
+    <t>PV of explicit FCF (mid-yr)</t>
   </si>
   <si>
     <t>Terminal Value</t>
@@ -513,6 +559,9 @@
     <t>PV of Terminal Value</t>
   </si>
   <si>
+    <t>FCF Yield (UFCF/EV)</t>
+  </si>
+  <si>
     <t>Enterprise Value (DCF)</t>
   </si>
   <si>
@@ -703,6 +752,78 @@
   </si>
   <si>
     <t>KPI Values →</t>
+  </si>
+  <si>
+    <t>COMPARABLE COMPANIES  (live peer multiples → implied value)</t>
+  </si>
+  <si>
+    <t>Mkt Cap ($M)</t>
+  </si>
+  <si>
+    <t>EV ($M)</t>
+  </si>
+  <si>
+    <t>EV/Rev (NTM)</t>
+  </si>
+  <si>
+    <t>EV/EBITDA (NTM)</t>
+  </si>
+  <si>
+    <t>P/E (NTM)</t>
+  </si>
+  <si>
+    <t>CRWD</t>
+  </si>
+  <si>
+    <t>PANW</t>
+  </si>
+  <si>
+    <t>ZS</t>
+  </si>
+  <si>
+    <t>NET</t>
+  </si>
+  <si>
+    <t>DDOG</t>
+  </si>
+  <si>
+    <t>SNOW</t>
+  </si>
+  <si>
+    <t>MDB</t>
+  </si>
+  <si>
+    <t>OKTA</t>
+  </si>
+  <si>
+    <t>Peer Median</t>
+  </si>
+  <si>
+    <t>IMPLIED VALUE — peer median × our consensus metric</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>Median ×</t>
+  </si>
+  <si>
+    <t>Our Metric ($M)</t>
+  </si>
+  <si>
+    <t>Implied ($M)</t>
+  </si>
+  <si>
+    <t>Implied Price</t>
+  </si>
+  <si>
+    <t>EV/Revenue</t>
+  </si>
+  <si>
+    <t>Average Implied</t>
+  </si>
+  <si>
+    <t>Comps populate in CapIQ mode (--capiq). Tickers shown are the sector-default peer set.</t>
   </si>
 </sst>
 </file>
@@ -711,12 +832,12 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="7">
     <numFmt numFmtId="164" formatCode="$#,##0.0"/>
-    <numFmt numFmtId="165" formatCode="$#,##0.00"/>
-    <numFmt numFmtId="166" formatCode="0.0&quot;x&quot;"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
-    <numFmt numFmtId="168" formatCode="#,##0"/>
-    <numFmt numFmtId="169" formatCode="MMM D, YYYY"/>
-    <numFmt numFmtId="170" formatCode="#,##0.0"/>
+    <numFmt numFmtId="168" formatCode="0.0&quot;x&quot;"/>
+    <numFmt numFmtId="169" formatCode="#,##0"/>
+    <numFmt numFmtId="170" formatCode="MMM D, YYYY"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -733,17 +854,7 @@
     </font>
     <font>
       <b/>
-    </font>
-    <font>
-      <b/>
       <color rgb="FFFFFFFF"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF2E5C9A"/>
-    </font>
-    <font>
-      <color rgb="FF1A1A1A"/>
     </font>
     <font>
       <b/>
@@ -752,7 +863,9 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF2E5C9A"/>
+    </font>
+    <font>
+      <color rgb="FF1A1A1A"/>
     </font>
     <font>
       <b/>
@@ -760,11 +873,27 @@
       <color rgb="FF2E5C9A"/>
     </font>
     <font>
+      <b/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF2E5C9A"/>
+    </font>
+    <font>
       <b val="0"/>
     </font>
     <font>
       <b/>
-      <sz val="14"/>
+      <color rgb="FF2E5C9A"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF9C6500"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
     </font>
     <font>
       <b/>
@@ -772,16 +901,8 @@
     </font>
     <font>
       <b/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <b/>
       <sz val="9"/>
       <color rgb="FFFFFFFF"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF9C6500"/>
     </font>
   </fonts>
   <fills count="9">
@@ -805,20 +926,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F6FC"/>
-        <bgColor rgb="FFF2F6FC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFD9E1F2"/>
         <bgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor rgb="FFC6EFCE"/>
+        <fgColor rgb="FFF2F6FC"/>
+        <bgColor rgb="FFF2F6FC"/>
       </patternFill>
     </fill>
     <fill>
@@ -831,6 +946,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
         <bgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -854,90 +975,106 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="170" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="13" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="167" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="168" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="170" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="11" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="168" fontId="13" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="13" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1505,395 +1642,395 @@
       <c r="L1" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="28" t="s">
         <v>1</v>
       </c>
       <c r="B3" t="str">
         <f>Inputs!D4</f>
         <v>Nimbus Cloud Inc</v>
       </c>
-      <c r="E3" s="20" t="s">
+      <c r="E3" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="48" t="s">
+      <c r="G3" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="20" t="s">
+      <c r="I3" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="J3" s="44">
+      <c r="J3" s="35">
         <f>Price</f>
         <v>45</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="28" t="s">
         <v>5</v>
       </c>
       <c r="B4" t="str">
         <f>Inputs!D5</f>
         <v>NIMB</v>
       </c>
-      <c r="E4" s="20" t="s">
+      <c r="E4" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="39">
+      <c r="F4" s="31">
         <f>Inputs!D10</f>
         <v>46231</v>
       </c>
-      <c r="I4" s="20" t="s">
+      <c r="I4" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="29">
+      <c r="J4" s="24">
         <f>Shares</f>
         <v>100</v>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="40" t="s">
+      <c r="B6" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="40"/>
-      <c r="D6" s="40"/>
-      <c r="F6" s="40" t="s">
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="F6" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="40"/>
-      <c r="H6" s="40"/>
-      <c r="J6" s="40" t="s">
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="J6" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="K6" s="40"/>
-      <c r="L6" s="40"/>
+      <c r="K6" s="20"/>
+      <c r="L6" s="20"/>
     </row>
     <row r="7">
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="35">
+      <c r="C7" s="26">
         <f>RevMy</f>
         <v>1160</v>
       </c>
-      <c r="D7" s="12"/>
-      <c r="F7" s="33" t="s">
+      <c r="D7" s="14"/>
+      <c r="F7" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="35">
+      <c r="G7" s="26">
         <f>EbitdaMy</f>
         <v>301.6</v>
       </c>
-      <c r="H7" s="12"/>
-      <c r="J7" s="33" t="s">
+      <c r="H7" s="14"/>
+      <c r="J7" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="K7" s="35">
+      <c r="K7" s="26">
         <f>NiMy</f>
         <v>156.60000000000002</v>
       </c>
-      <c r="L7" s="12"/>
+      <c r="L7" s="14"/>
     </row>
     <row r="8">
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="35">
+      <c r="C8" s="26">
         <f>ConsRev</f>
         <v>1150</v>
       </c>
-      <c r="D8" s="12"/>
-      <c r="F8" s="33" t="s">
+      <c r="D8" s="14"/>
+      <c r="F8" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="35">
+      <c r="G8" s="26">
         <f>ConsEBITDA</f>
         <v>295</v>
       </c>
-      <c r="H8" s="12"/>
-      <c r="J8" s="33" t="s">
+      <c r="H8" s="14"/>
+      <c r="J8" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="K8" s="35">
+      <c r="K8" s="26">
         <f>ConsNI</f>
         <v>150</v>
       </c>
-      <c r="L8" s="12"/>
+      <c r="L8" s="14"/>
     </row>
     <row r="9">
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="31">
+      <c r="C9" s="23">
         <f>RevMy/PriorRev-1</f>
         <v>0.15999999999999992</v>
       </c>
-      <c r="D9" s="12"/>
-      <c r="F9" s="33" t="s">
+      <c r="D9" s="14"/>
+      <c r="F9" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="31">
+      <c r="G9" s="23">
         <f>EbitdaMy/PriorEBITDA-1</f>
         <v>0.20640000000000014</v>
       </c>
-      <c r="H9" s="12"/>
-      <c r="J9" s="33" t="s">
+      <c r="H9" s="14"/>
+      <c r="J9" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="K9" s="31">
+      <c r="K9" s="23">
         <f>NiMy/PriorNI-1</f>
         <v>0.30500000000000016</v>
       </c>
-      <c r="L9" s="12"/>
+      <c r="L9" s="14"/>
     </row>
     <row r="10">
-      <c r="B10" s="33" t="s">
+      <c r="B10" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="31">
+      <c r="C10" s="23">
         <f>RevMy/ConsRev-1</f>
         <v>0.008695652173912993</v>
       </c>
-      <c r="D10" s="12"/>
-      <c r="F10" s="33" t="s">
+      <c r="D10" s="14"/>
+      <c r="F10" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="31">
+      <c r="G10" s="23">
         <f>EbitdaMy/ConsEBITDA-1</f>
         <v>0.022372881355932295</v>
       </c>
-      <c r="H10" s="12"/>
-      <c r="J10" s="33" t="s">
+      <c r="H10" s="14"/>
+      <c r="J10" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K10" s="31">
+      <c r="K10" s="23">
         <f>NiMy/ConsNI-1</f>
         <v>0.04400000000000026</v>
       </c>
-      <c r="L10" s="12"/>
+      <c r="L10" s="14"/>
     </row>
     <row r="11">
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="38" t="str">
+      <c r="C11" s="30" t="str">
         <f>IF(RevMy/ConsRev-1&gt;=BeatThresh,"BEAT",IF(RevMy/ConsRev-1&lt;=MissThresh,"MISS","IN-LINE"))</f>
         <v>IN-LINE</v>
       </c>
-      <c r="D11" s="12"/>
-      <c r="F11" s="33" t="s">
+      <c r="D11" s="14"/>
+      <c r="F11" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="G11" s="38" t="str">
+      <c r="G11" s="30" t="str">
         <f>IF(EbitdaMy/ConsEBITDA-1&gt;=BeatThresh,"BEAT",IF(EbitdaMy/ConsEBITDA-1&lt;=MissThresh,"MISS","IN-LINE"))</f>
         <v>BEAT</v>
       </c>
-      <c r="H11" s="12"/>
-      <c r="J11" s="33" t="s">
+      <c r="H11" s="14"/>
+      <c r="J11" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="K11" s="38" t="str">
+      <c r="K11" s="30" t="str">
         <f>IF(NiMy/ConsNI-1&gt;=BeatThresh,"BEAT",IF(NiMy/ConsNI-1&lt;=MissThresh,"MISS","IN-LINE"))</f>
         <v>BEAT</v>
       </c>
-      <c r="L11" s="12"/>
+      <c r="L11" s="14"/>
     </row>
     <row r="13">
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
-      <c r="K13" s="8"/>
-      <c r="L13" s="8"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
     </row>
     <row r="14">
-      <c r="B14" s="28" t="str">
+      <c r="B14" s="17" t="str">
         <f>INDEX(KpiNames,1,MATCH(SelectedSector,SectorList,0))</f>
         <v>ARR ($M)</v>
       </c>
-      <c r="C14" s="28"/>
-      <c r="D14" s="28" t="str">
+      <c r="C14" s="17"/>
+      <c r="D14" s="17" t="str">
         <f>INDEX(KpiNames,2,MATCH(SelectedSector,SectorList,0))</f>
         <v>Net Rev Retention (%)</v>
       </c>
-      <c r="E14" s="28"/>
-      <c r="F14" s="28" t="str">
+      <c r="E14" s="17"/>
+      <c r="F14" s="17" t="str">
         <f>INDEX(KpiNames,3,MATCH(SelectedSector,SectorList,0))</f>
         <v>Rule of 40 (%)</v>
       </c>
-      <c r="G14" s="28"/>
-      <c r="H14" s="28" t="str">
+      <c r="G14" s="17"/>
+      <c r="H14" s="17" t="str">
         <f>INDEX(KpiNames,4,MATCH(SelectedSector,SectorList,0))</f>
         <v>Gross Margin (%)</v>
       </c>
-      <c r="I14" s="28"/>
-      <c r="J14" s="28" t="str">
+      <c r="I14" s="17"/>
+      <c r="J14" s="17" t="str">
         <f>INDEX(KpiNames,5,MATCH(SelectedSector,SectorList,0))</f>
         <v>CAC Payback (mo)</v>
       </c>
-      <c r="K14" s="28"/>
+      <c r="K14" s="17"/>
     </row>
     <row r="15">
-      <c r="B15" s="36">
+      <c r="B15" s="18">
         <f>INDEX(KpiValues,1,MATCH(SelectedSector,SectorList,0))</f>
         <v>1200</v>
       </c>
-      <c r="C15" s="36"/>
-      <c r="D15" s="36">
+      <c r="C15" s="18"/>
+      <c r="D15" s="18">
         <f>INDEX(KpiValues,2,MATCH(SelectedSector,SectorList,0))</f>
         <v>118</v>
       </c>
-      <c r="E15" s="36"/>
-      <c r="F15" s="36">
+      <c r="E15" s="18"/>
+      <c r="F15" s="18">
         <f>INDEX(KpiValues,3,MATCH(SelectedSector,SectorList,0))</f>
         <v>46</v>
       </c>
-      <c r="G15" s="36"/>
-      <c r="H15" s="36">
+      <c r="G15" s="18"/>
+      <c r="H15" s="18">
         <f>INDEX(KpiValues,4,MATCH(SelectedSector,SectorList,0))</f>
         <v>78</v>
       </c>
-      <c r="I15" s="36"/>
-      <c r="J15" s="36">
+      <c r="I15" s="18"/>
+      <c r="J15" s="18">
         <f>INDEX(KpiValues,5,MATCH(SelectedSector,SectorList,0))</f>
         <v>14</v>
       </c>
-      <c r="K15" s="36"/>
+      <c r="K15" s="18"/>
     </row>
     <row r="17">
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
-      <c r="K17" s="8"/>
-      <c r="L17" s="8"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="6"/>
+      <c r="K17" s="6"/>
+      <c r="L17" s="6"/>
     </row>
     <row r="18">
-      <c r="B18" s="32" t="s">
+      <c r="B18" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="32" t="s">
+      <c r="C18" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D18" s="32" t="s">
+      <c r="D18" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="E18" s="32" t="s">
+      <c r="E18" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="F18" s="32" t="s">
+      <c r="F18" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="G18" s="32" t="s">
+      <c r="G18" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="H18" s="32" t="s">
+      <c r="H18" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="I18" s="32" t="s">
+      <c r="I18" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="J18" s="32" t="s">
+      <c r="J18" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="K18" s="32" t="s">
+      <c r="K18" s="13" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="45">
+      <c r="B19" s="21">
         <f>Valuation!C5</f>
         <v>14.423076923076922</v>
       </c>
-      <c r="C19" s="45">
+      <c r="C19" s="21">
         <f>Valuation!C6</f>
         <v>28.73563218390804</v>
       </c>
-      <c r="D19" s="45">
+      <c r="D19" s="21">
         <f>Valuation!C7</f>
         <v>3.75</v>
       </c>
-      <c r="E19" s="45">
+      <c r="E19" s="21">
         <f>Valuation!C8</f>
         <v>3.8793103448275863</v>
       </c>
-      <c r="F19" s="34">
+      <c r="F19" s="16">
         <f>FairValue</f>
-        <v>45.85775303860559</v>
-      </c>
-      <c r="G19" s="34">
+        <v>44.293140480958506</v>
+      </c>
+      <c r="G19" s="16">
         <f>DcfExit</f>
-        <v>52.536521739254994</v>
-      </c>
-      <c r="H19" s="34">
+        <v>59.5519499119956</v>
+      </c>
+      <c r="H19" s="16">
         <f>ValMid</f>
         <v>48.165</v>
       </c>
-      <c r="I19" s="34">
+      <c r="I19" s="16">
         <f>AvgImplied</f>
         <v>48.165</v>
       </c>
-      <c r="J19" s="34">
+      <c r="J19" s="16">
         <f>Price</f>
         <v>45</v>
       </c>
-      <c r="K19" s="46">
+      <c r="K19" s="39">
         <f>Valuation!J24</f>
         <v>0.07033333333333336</v>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
-      <c r="K21" s="8"/>
-      <c r="L21" s="8"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="6"/>
+      <c r="K21" s="6"/>
+      <c r="L21" s="6"/>
     </row>
     <row r="22">
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="D22" s="41">
+      <c r="D22" s="32">
         <f>AVERAGE(RevMy/ConsRev-1,EbitdaMy/ConsEBITDA-1,NiMy/ConsNI-1)</f>
         <v>0.025022844509948516</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="F22" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="H22" s="43" t="str">
+      <c r="H22" s="34" t="str">
         <f>IF(D22&gt;=BeatThresh,"LIKELY BEAT  ▲",IF(D22&lt;=MissThresh,"LIKELY MISS  ▼","IN-LINE  ►"))</f>
         <v>LIKELY BEAT  ▲</v>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="D23" s="41">
+      <c r="D23" s="32">
         <f>D22*ReactSens</f>
         <v>0.20018275607958813</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="F23" s="15" t="s">
         <v>30</v>
       </c>
       <c r="H23" t="str">
@@ -1902,23 +2039,23 @@
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="19" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="47" t="s">
+      <c r="B43" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="C43" s="47" t="s">
+      <c r="C43" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="D43" s="47" t="s">
+      <c r="D43" s="40" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="3" t="s">
+      <c r="B44" s="15" t="s">
         <v>34</v>
       </c>
       <c r="C44" s="1">
@@ -1931,7 +2068,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="B45" s="3" t="s">
+      <c r="B45" s="15" t="s">
         <v>35</v>
       </c>
       <c r="C45" s="1">
@@ -1944,7 +2081,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="3" t="s">
+      <c r="B46" s="15" t="s">
         <v>36</v>
       </c>
       <c r="C46" s="1">
@@ -1958,41 +2095,41 @@
     </row>
   </sheetData>
   <mergeCells count="35">
+    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="H23:L23"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="A1:L1"/>
     <mergeCell ref="D14:E14"/>
+    <mergeCell ref="B21:L21"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="K8:L8"/>
     <mergeCell ref="G11:H11"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="K11:L11"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B17:L17"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="B13:L13"/>
+    <mergeCell ref="H15:I15"/>
     <mergeCell ref="H22:L22"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="J6:L6"/>
     <mergeCell ref="B40:L40"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="B13:L13"/>
-    <mergeCell ref="F6:H6"/>
-    <mergeCell ref="B17:L17"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="C7:D7"/>
     <mergeCell ref="F14:G14"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J14:K14"/>
     <mergeCell ref="G7:H7"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="B21:L21"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="F15:G15"/>
     <mergeCell ref="H14:I14"/>
-    <mergeCell ref="K8:L8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="H23:L23"/>
-    <mergeCell ref="K10:L10"/>
-    <mergeCell ref="K11:L11"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="B6:D6"/>
   </mergeCells>
   <conditionalFormatting sqref="H22">
     <cfRule type="expression" dxfId="0" priority="1">
@@ -2113,7 +2250,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr defaultColWidth="8.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.5703125" customWidth="1"/>
@@ -2135,70 +2272,70 @@
       <c r="F1" s="2"/>
     </row>
     <row r="3">
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="F3" s="8" t="s">
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="F3" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
     </row>
     <row r="4">
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="19" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="14" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="53">
         <v>45</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="I6" s="11" t="s">
+      <c r="I6" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="J6" s="11" t="s">
+      <c r="J6" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="K6" s="11" t="s">
+      <c r="K6" s="8" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="48" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="54">
         <v>100</v>
       </c>
       <c r="F7" t="s">
@@ -2213,7 +2350,7 @@
       <c r="I7" s="5">
         <v>45</v>
       </c>
-      <c r="J7" s="14">
+      <c r="J7" s="50">
         <v>100</v>
       </c>
       <c r="K7" s="1">
@@ -2221,10 +2358,10 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="48" t="s">
         <v>48</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="51">
         <v>-150</v>
       </c>
       <c r="F8" t="s">
@@ -2239,7 +2376,7 @@
       <c r="I8" s="5">
         <v>62</v>
       </c>
-      <c r="J8" s="14">
+      <c r="J8" s="50">
         <v>210</v>
       </c>
       <c r="K8" s="1">
@@ -2247,10 +2384,10 @@
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="49">
         <v>0.21</v>
       </c>
       <c r="F9" t="s">
@@ -2265,7 +2402,7 @@
       <c r="I9" s="5">
         <v>95</v>
       </c>
-      <c r="J9" s="14">
+      <c r="J9" s="50">
         <v>400</v>
       </c>
       <c r="K9" s="1">
@@ -2273,260 +2410,332 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="48" t="s">
         <v>56</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="56">
         <v>46231</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="48" t="s">
         <v>57</v>
       </c>
-      <c r="D11" s="12" t="str">
+      <c r="D11" s="14" t="str">
         <f>SelectedSector</f>
         <v>Tech/SaaS</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
     </row>
     <row r="14">
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="48" t="s">
         <v>59</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="49">
         <v>0.16</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="48" t="s">
         <v>60</v>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="49">
         <v>0.03</v>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="48" t="s">
         <v>61</v>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="49">
         <v>0.26</v>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="48" t="s">
         <v>62</v>
       </c>
-      <c r="D17" s="10">
+      <c r="D17" s="49">
         <v>0.135</v>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="48" t="s">
         <v>63</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="49">
         <v>0.85</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="48" t="s">
         <v>64</v>
       </c>
-      <c r="D19" s="12" t="s">
+      <c r="D19" s="14" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="48" t="s">
         <v>66</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="55">
         <f>IF(ScenarioName="Bull",1.25,IF(ScenarioName="Bear",0.7,1))</f>
         <v>1</v>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
     </row>
     <row r="23">
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="48" t="s">
         <v>68</v>
       </c>
-      <c r="D23" s="9">
+      <c r="D23" s="55">
         <v>13</v>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="48" t="s">
         <v>69</v>
       </c>
-      <c r="D24" s="9">
+      <c r="D24" s="55">
         <v>22</v>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="48" t="s">
         <v>70</v>
       </c>
-      <c r="D25" s="9">
+      <c r="D25" s="55">
         <v>5</v>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="48" t="s">
         <v>71</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="55">
         <v>5</v>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
     </row>
     <row r="29">
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="48" t="s">
         <v>73</v>
       </c>
-      <c r="D29" s="10">
+      <c r="D29" s="49">
         <v>0.042</v>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="D30" s="10">
+      <c r="D30" s="49">
         <v>0.05</v>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="7" t="s">
+      <c r="B31" s="48" t="s">
         <v>75</v>
       </c>
-      <c r="D31" s="17">
+      <c r="D31" s="52">
         <v>1.2</v>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="7" t="s">
+      <c r="B32" s="48" t="s">
         <v>76</v>
       </c>
-      <c r="D32" s="10">
+      <c r="D32" s="49">
         <v>0.06</v>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="7" t="s">
+      <c r="B33" s="48" t="s">
         <v>77</v>
       </c>
-      <c r="D33" s="10">
+      <c r="D33" s="49">
         <v>0.85</v>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="48" t="s">
         <v>78</v>
       </c>
-      <c r="D34" s="10">
+      <c r="D34" s="49">
         <v>0.15</v>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="7" t="s">
+      <c r="B35" s="48" t="s">
         <v>79</v>
       </c>
-      <c r="D35" s="10">
+      <c r="D35" s="49">
         <v>0.03</v>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="8" t="s">
+      <c r="B37" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="C37" s="8"/>
-      <c r="D37" s="8"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
     </row>
     <row r="38">
-      <c r="B38" s="7" t="s">
+      <c r="B38" s="48" t="s">
         <v>81</v>
       </c>
-      <c r="D38" s="10">
+      <c r="D38" s="49">
         <v>0.02</v>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="7" t="s">
+      <c r="B39" s="48" t="s">
         <v>82</v>
       </c>
-      <c r="D39" s="10">
+      <c r="D39" s="49">
         <v>-0.02</v>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="7" t="s">
+      <c r="B40" s="48" t="s">
         <v>83</v>
       </c>
-      <c r="D40" s="9">
+      <c r="D40" s="55">
         <v>8</v>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="8" t="s">
+      <c r="B42" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="C42" s="8"/>
-      <c r="D42" s="8"/>
+      <c r="C42" s="6"/>
+      <c r="D42" s="6"/>
     </row>
     <row r="43">
-      <c r="B43" s="7" t="s">
+      <c r="B43" s="48" t="s">
         <v>85</v>
       </c>
-      <c r="D43" s="13"/>
+      <c r="D43" s="53"/>
     </row>
     <row r="44">
-      <c r="B44" s="7" t="s">
+      <c r="B44" s="48" t="s">
         <v>86</v>
       </c>
-      <c r="D44" s="15"/>
+      <c r="D44" s="51"/>
     </row>
     <row r="45">
-      <c r="B45" s="7" t="s">
+      <c r="B45" s="48" t="s">
         <v>87</v>
       </c>
-      <c r="D45" s="13"/>
+      <c r="D45" s="53"/>
     </row>
     <row r="46">
-      <c r="B46" s="7" t="s">
+      <c r="B46" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="D46" s="12"/>
+      <c r="D46" s="14"/>
+    </row>
+    <row r="51">
+      <c r="B51" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="C51" s="6"/>
+      <c r="D51" s="6"/>
+    </row>
+    <row r="52">
+      <c r="B52" s="48" t="s">
+        <v>90</v>
+      </c>
+      <c r="D52" s="49">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="48" t="s">
+        <v>91</v>
+      </c>
+      <c r="D53" s="49">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="48" t="s">
+        <v>92</v>
+      </c>
+      <c r="D54" s="49">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="48" t="s">
+        <v>93</v>
+      </c>
+      <c r="D55" s="49">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="48" t="s">
+        <v>94</v>
+      </c>
+      <c r="D56" s="49">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="48" t="s">
+        <v>95</v>
+      </c>
+      <c r="D57" s="54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="48" t="s">
+        <v>96</v>
+      </c>
+      <c r="D58" s="51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="48" t="s">
+        <v>97</v>
+      </c>
+      <c r="D59" s="51">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="B42:D42"/>
+    <mergeCell ref="A1:F1"/>
     <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="B51:D51"/>
+    <mergeCell ref="F3:K3"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B28:D28"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="F3:K3"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B28:D28"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D19">
@@ -2548,7 +2757,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2557,20 +2766,20 @@
     </row>
     <row r="3">
       <c r="B3" s="4" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="15" t="s">
         <v>34</v>
       </c>
       <c r="C4" s="1">
@@ -2584,7 +2793,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="15" t="s">
         <v>35</v>
       </c>
       <c r="C5" s="1">
@@ -2598,7 +2807,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="15" t="s">
         <v>36</v>
       </c>
       <c r="C6" s="1">
@@ -2612,8 +2821,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="3" t="s">
-        <v>94</v>
+      <c r="B7" s="15" t="s">
+        <v>103</v>
       </c>
       <c r="C7" s="5">
         <f>C6/Shares</f>
@@ -2648,7 +2857,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2656,73 +2865,73 @@
     </row>
     <row r="3">
       <c r="B3" s="4" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="15" t="s">
         <v>34</v>
       </c>
       <c r="C4" s="1">
         <f>PriorRev*(1+RevGrowthMy*ScenarioMult)</f>
         <v>1160</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>98</v>
+      <c r="D4" s="19" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="15" t="s">
         <v>35</v>
       </c>
       <c r="C5" s="1">
         <f>RevMy*EbitdaMarginMy</f>
         <v>301.6</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>99</v>
+      <c r="D5" s="19" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="15" t="s">
         <v>36</v>
       </c>
       <c r="C6" s="1">
         <f>RevMy*NiMarginMy</f>
         <v>156.60000000000002</v>
       </c>
-      <c r="D6" s="6" t="s">
-        <v>100</v>
+      <c r="D6" s="19" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="3" t="s">
-        <v>94</v>
+      <c r="B7" s="15" t="s">
+        <v>103</v>
       </c>
       <c r="C7" s="5">
         <f>NiMy/Shares</f>
         <v>1.5660000000000003</v>
       </c>
-      <c r="D7" s="6" t="s">
-        <v>101</v>
+      <c r="D7" s="19" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="3" t="s">
-        <v>102</v>
+      <c r="B8" s="15" t="s">
+        <v>111</v>
       </c>
       <c r="C8" s="1">
         <f>EbitdaMy*(1-TaxRate)*FcfConv</f>
         <v>202.5244</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>103</v>
+      <c r="D8" s="19" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -2747,7 +2956,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2758,288 +2967,288 @@
       <c r="H1" s="2"/>
     </row>
     <row r="3">
-      <c r="B3" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="C3" s="8"/>
-      <c r="I3" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
+      <c r="B3" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C3" s="6"/>
+      <c r="I3" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
     </row>
     <row r="4">
       <c r="B4" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="C4" s="1">
-        <f>Price*Shares+NetDebt</f>
+        <f>Price*Shares+NetDebt+Minorities-Associates</f>
         <v>4350</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="s">
-        <v>108</v>
-      </c>
-      <c r="C5" s="25">
+        <v>117</v>
+      </c>
+      <c r="C5" s="11">
         <f>EV/EbitdaMy</f>
         <v>14.423076923076922</v>
       </c>
-      <c r="I5" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="J5" s="11" t="s">
-        <v>110</v>
+      <c r="I5" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="s">
-        <v>111</v>
-      </c>
-      <c r="C6" s="25">
+        <v>120</v>
+      </c>
+      <c r="C6" s="11">
         <f>Price/EpsMy</f>
         <v>28.73563218390804</v>
       </c>
       <c r="I6" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="J6" s="1">
         <f>C30</f>
-        <v>5245.320977081592</v>
+        <v>4974.535242201786</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="s">
-        <v>113</v>
-      </c>
-      <c r="C7" s="25">
+        <v>122</v>
+      </c>
+      <c r="C7" s="11">
         <f>EV/RevMy</f>
         <v>3.75</v>
       </c>
       <c r="I7" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="J7" s="1">
         <f>G26*PeerEVEBITDA</f>
-        <v>6291.0179501311995</v>
+        <v>7258.866865536</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="s">
-        <v>115</v>
-      </c>
-      <c r="C8" s="25">
+        <v>124</v>
+      </c>
+      <c r="C8" s="11">
         <f>Price*Shares/RevMy</f>
         <v>3.8793103448275863</v>
       </c>
       <c r="I8" t="s">
-        <v>116</v>
-      </c>
-      <c r="J8" s="25">
+        <v>125</v>
+      </c>
+      <c r="J8" s="11">
         <f>C30/G26</f>
-        <v>10.839131797523898</v>
+        <v>8.908960495702384</v>
       </c>
     </row>
     <row r="9">
       <c r="I9" t="s">
-        <v>117</v>
-      </c>
-      <c r="J9" s="23">
+        <v>126</v>
+      </c>
+      <c r="J9" s="7">
         <f>(WACC*J7-G27)/(J7+G27)</f>
-        <v>0.04008557949018031</v>
+        <v>0.04926289201078474</v>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="C10" s="8"/>
+      <c r="B10" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C10" s="6"/>
     </row>
     <row r="11">
       <c r="B11" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="C11" s="5">
         <f>(PeerEVEBITDA*EbitdaMy-NetDebt)/Shares</f>
         <v>40.708</v>
       </c>
-      <c r="I11" s="11" t="s">
-        <v>120</v>
-      </c>
-      <c r="J11" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="K11" s="11" t="s">
-        <v>121</v>
+      <c r="I11" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="C12" s="5">
         <f>PeerPE*EpsMy</f>
         <v>34.452000000000005</v>
       </c>
       <c r="I12" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="J12" s="5">
         <f>FairValue</f>
-        <v>45.85775303860559</v>
-      </c>
-      <c r="K12" s="23">
+        <v>44.293140480958506</v>
+      </c>
+      <c r="K12" s="7">
         <f>IFERROR(J12/Price-1,"")</f>
-        <v>0.0190611786356798</v>
+        <v>-0.01570798931203321</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="C13" s="5">
         <f>(PeerEVRev*RevMy-NetDebt)/Shares</f>
         <v>59.5</v>
       </c>
       <c r="I13" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="J13" s="5">
-        <f>((C29+J7/(1+WACC)^5)-NetDebt)/Shares</f>
-        <v>52.536521739254994</v>
-      </c>
-      <c r="K13" s="23">
+        <f>((C29+J7/(1+WACC)^4.5)-NetDebt-Minorities+Associates)/Shares</f>
+        <v>59.5519499119956</v>
+      </c>
+      <c r="K13" s="7">
         <f>IFERROR(J13/Price-1,"")</f>
-        <v>0.16747826087233308</v>
+        <v>0.32337666471101323</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="C14" s="5">
         <f>PeerPS*RevMy/Shares</f>
         <v>58</v>
       </c>
       <c r="I14" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="J14" s="5">
         <f>AvgImplied</f>
         <v>48.165</v>
       </c>
-      <c r="K14" s="23">
+      <c r="K14" s="7">
         <f>IFERROR(J14/Price-1,"")</f>
         <v>0.07033333333333336</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="C15" s="42">
+      <c r="B15" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="C15" s="41">
         <f>AVERAGE(C11:C14)</f>
         <v>48.165</v>
       </c>
       <c r="I15" t="s">
-        <v>129</v>
-      </c>
-      <c r="K15" s="23"/>
+        <v>138</v>
+      </c>
+      <c r="K15" s="7"/>
     </row>
     <row r="17">
-      <c r="B17" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="C17" s="8"/>
+      <c r="B17" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="C17" s="6"/>
       <c r="I17" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="J17" s="5"/>
       <c r="K17" s="5"/>
     </row>
     <row r="18">
       <c r="B18" t="s">
-        <v>132</v>
-      </c>
-      <c r="C18" s="23">
+        <v>141</v>
+      </c>
+      <c r="C18" s="7">
         <f>RiskFree+Beta*ERP</f>
         <v>0.10200000000000001</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" t="s">
-        <v>133</v>
-      </c>
-      <c r="C19" s="23">
+        <v>142</v>
+      </c>
+      <c r="C19" s="7">
         <f>CostDebt*(1-TaxRate)</f>
         <v>0.0474</v>
       </c>
-      <c r="I19" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="J19" s="8"/>
-      <c r="K19" s="8"/>
+      <c r="I19" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="J19" s="6"/>
+      <c r="K19" s="6"/>
     </row>
     <row r="20">
-      <c r="B20" s="11" t="s">
-        <v>130</v>
-      </c>
-      <c r="C20" s="30">
+      <c r="B20" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="C20" s="22">
         <f>WeightEquity*C18+WeightDebt*C19</f>
         <v>0.09381</v>
       </c>
       <c r="I20" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="J20" s="5">
         <f>MIN(J12:J15)</f>
-        <v>45.85775303860559</v>
+        <v>44.293140480958506</v>
       </c>
     </row>
     <row r="21">
       <c r="I21" t="s">
-        <v>136</v>
-      </c>
-      <c r="J21" s="37">
+        <v>145</v>
+      </c>
+      <c r="J21" s="38">
         <f>MEDIAN(J12:J15)</f>
         <v>48.165</v>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
+      <c r="B22" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
       <c r="I22" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="J22" s="5">
         <f>MAX(J12:J15)</f>
-        <v>52.536521739254994</v>
+        <v>59.5519499119956</v>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="21" t="s">
-        <v>139</v>
-      </c>
-      <c r="C23" s="21">
+      <c r="B23" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="C23" s="10">
         <v>1</v>
       </c>
-      <c r="D23" s="21">
+      <c r="D23" s="10">
         <v>2</v>
       </c>
-      <c r="E23" s="21">
+      <c r="E23" s="10">
         <v>3</v>
       </c>
-      <c r="F23" s="21">
+      <c r="F23" s="10">
         <v>4</v>
       </c>
-      <c r="G23" s="21">
+      <c r="G23" s="10">
         <v>5</v>
       </c>
       <c r="I23" t="s">
@@ -3051,40 +3260,40 @@
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C24" s="23">
+      <c r="B24" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="C24" s="7">
         <f>MAX(RevGrowthMy*ScenarioMult,TermGrowth)</f>
         <v>0.16</v>
       </c>
-      <c r="D24" s="23">
+      <c r="D24" s="7">
         <f>MAX(C24-GrowthFade,TermGrowth)</f>
         <v>0.13</v>
       </c>
-      <c r="E24" s="23">
+      <c r="E24" s="7">
         <f>MAX(D24-GrowthFade,TermGrowth)</f>
         <v>0.1</v>
       </c>
-      <c r="F24" s="23">
+      <c r="F24" s="7">
         <f>MAX(E24-GrowthFade,TermGrowth)</f>
         <v>0.07</v>
       </c>
-      <c r="G24" s="23">
+      <c r="G24" s="7">
         <f>MAX(F24-GrowthFade,TermGrowth)</f>
         <v>0.04000000000000001</v>
       </c>
       <c r="I24" t="s">
-        <v>141</v>
-      </c>
-      <c r="J24" s="26">
+        <v>150</v>
+      </c>
+      <c r="J24" s="37">
         <f>J21/Price-1</f>
         <v>0.07033333333333336</v>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="3" t="s">
-        <v>142</v>
+      <c r="B25" s="15" t="s">
+        <v>151</v>
       </c>
       <c r="C25" s="1">
         <f>RevMy*(1+C24)</f>
@@ -3108,132 +3317,192 @@
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="15" t="s">
         <v>9</v>
       </c>
       <c r="C26" s="1">
-        <f>C25*EbitdaMarginMy</f>
+        <f>C25*(EbitdaMarginMy+(TermMargin-EbitdaMarginMy)*0)</f>
         <v>349.856</v>
       </c>
       <c r="D26" s="1">
-        <f>D25*EbitdaMarginMy</f>
-        <v>395.33727999999996</v>
+        <f>D25*(EbitdaMarginMy+(TermMargin-EbitdaMarginMy)*0.25)</f>
+        <v>410.54256</v>
       </c>
       <c r="E26" s="1">
-        <f>E25*EbitdaMarginMy</f>
-        <v>434.871008</v>
+        <f>E25*(EbitdaMarginMy+(TermMargin-EbitdaMarginMy)*0.5)</f>
+        <v>468.322624</v>
       </c>
       <c r="F26" s="1">
-        <f>F25*EbitdaMarginMy</f>
-        <v>465.31197856</v>
+        <f>F25*(EbitdaMarginMy+(TermMargin-EbitdaMarginMy)*0.75)</f>
+        <v>519.00182224</v>
       </c>
       <c r="G26" s="1">
-        <f>G25*EbitdaMarginMy</f>
-        <v>483.9244577024</v>
-      </c>
+        <f>G25*(EbitdaMarginMy+(TermMargin-EbitdaMarginMy)*1)</f>
+        <v>558.374374272</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="J26" s="6"/>
+      <c r="K26" s="6"/>
     </row>
     <row r="27">
-      <c r="B27" s="3" t="s">
-        <v>143</v>
+      <c r="B27" s="15" t="s">
+        <v>153</v>
       </c>
       <c r="C27" s="1">
-        <f>C26*(1-TaxRate)*FcfConv</f>
-        <v>234.92830399999997</v>
+        <f>C26-C25*CapexPct-MAX(C26-C25*DaPct,0)*TaxRate-(C25-RevMy)*NwcPct-IF(SbcDeduct=1,C25*SbcPct,0)</f>
+        <v>173.58704000000003</v>
       </c>
       <c r="D27" s="1">
-        <f>D26*(1-TaxRate)*FcfConv</f>
-        <v>265.46898351999994</v>
+        <f>D26-D25*CapexPct-MAX(D26-D25*DaPct,0)*TaxRate-(D25-C25)*NwcPct-IF(SbcDeduct=1,D25*SbcPct,0)</f>
+        <v>209.90552640000004</v>
       </c>
       <c r="E27" s="1">
-        <f>E26*(1-TaxRate)*FcfConv</f>
-        <v>292.015881872</v>
+        <f>E26-E25*CapexPct-MAX(E26-E25*DaPct,0)*TaxRate-(E25-D25)*NwcPct-IF(SbcDeduct=1,E25*SbcPct,0)</f>
+        <v>246.12786736</v>
       </c>
       <c r="F27" s="1">
-        <f>F26*(1-TaxRate)*FcfConv</f>
-        <v>312.45699360304</v>
+        <f>F26-F25*CapexPct-MAX(F26-F25*DaPct,0)*TaxRate-(F25-E25)*NwcPct-IF(SbcDeduct=1,F25*SbcPct,0)</f>
+        <v>279.77593557759997</v>
       </c>
       <c r="G27" s="1">
-        <f>G26*(1-TaxRate)*FcfConv</f>
-        <v>324.95527334716155</v>
+        <f>G26-G25*CapexPct-MAX(G26-G25*DaPct,0)*TaxRate-(G25-F25)*NwcPct-IF(SbcDeduct=1,G25*SbcPct,0)</f>
+        <v>308.17970272319997</v>
+      </c>
+      <c r="I27" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="J27" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="K27" s="8" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="I28" t="s">
+        <v>122</v>
+      </c>
+      <c r="J28" s="33">
+        <f>EV/ConsRev</f>
+        <v>3.782608695652174</v>
+      </c>
+      <c r="K28" s="33">
+        <f>EV/Consensus!E4</f>
+        <v>3.3461538461538463</v>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="C29" s="1">
-        <f>NPV(WACC,C27:G27)</f>
-        <v>1085.6378864760316</v>
+        <f>NPV(WACC,C27:G27)*(1+WACC)^0.5</f>
+        <v>956.4390113293764</v>
+      </c>
+      <c r="I29" t="s">
+        <v>117</v>
+      </c>
+      <c r="J29" s="33">
+        <f>EV/ConsEBITDA</f>
+        <v>14.745762711864407</v>
+      </c>
+      <c r="K29" s="33">
+        <f>EV/Consensus!E5</f>
+        <v>12.794117647058824</v>
       </c>
     </row>
     <row r="30">
       <c r="B30" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="C30" s="1">
         <f>G27*(1+TermGrowth)/(WACC-TermGrowth)</f>
-        <v>5245.320977081592</v>
+        <v>4974.535242201786</v>
+      </c>
+      <c r="I30" t="s">
+        <v>120</v>
+      </c>
+      <c r="J30" s="33">
+        <f>Price*Shares/ConsNI</f>
+        <v>30</v>
+      </c>
+      <c r="K30" s="33">
+        <f>Price*Shares/Consensus!E6</f>
+        <v>25.714285714285715</v>
       </c>
     </row>
     <row r="31">
       <c r="B31" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="C31" s="1">
-        <f>C30/(1+WACC)^5</f>
-        <v>3350.137417384527</v>
+        <f>C30/(1+WACC)^4.5</f>
+        <v>3322.8750367664748</v>
+      </c>
+      <c r="I31" t="s">
+        <v>159</v>
+      </c>
+      <c r="J31" s="25">
+        <f>C27/EV</f>
+        <v>0.039905066666666676</v>
+      </c>
+      <c r="K31" s="25">
+        <f>G27/EV</f>
+        <v>0.070845908672</v>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="3" t="s">
-        <v>147</v>
+      <c r="B32" s="15" t="s">
+        <v>160</v>
       </c>
       <c r="C32" s="1">
         <f>C29+C31</f>
-        <v>4435.775303860559</v>
+        <v>4279.314048095851</v>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="3" t="s">
-        <v>148</v>
+      <c r="B33" s="15" t="s">
+        <v>161</v>
       </c>
       <c r="C33" s="1">
-        <f>C32-NetDebt</f>
-        <v>4585.775303860559</v>
+        <f>C32-NetDebt-Minorities+Associates</f>
+        <v>4429.314048095851</v>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C34" s="37">
+      <c r="B34" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C34" s="38">
         <f>C33/Shares</f>
-        <v>45.85775303860559</v>
+        <v>44.293140480958506</v>
       </c>
     </row>
     <row r="35">
       <c r="B35" t="s">
-        <v>149</v>
-      </c>
-      <c r="C35" s="26">
+        <v>162</v>
+      </c>
+      <c r="C35" s="37">
         <f>FairValue/Price-1</f>
-        <v>0.0190611786356798</v>
+        <v>-0.01570798931203321</v>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C37" s="8"/>
-      <c r="D37" s="8"/>
-      <c r="E37" s="8"/>
-      <c r="F37" s="8"/>
-      <c r="G37" s="8"/>
-      <c r="H37" s="8"/>
+      <c r="B37" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
     </row>
     <row r="38">
       <c r="B38" s="27" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="C38" s="27">
         <f>TermGrowth+-0.01</f>
@@ -3257,145 +3526,146 @@
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="30">
+      <c r="B39" s="22">
         <f>WACC+-0.01</f>
         <v>0.08381000000000001</v>
       </c>
-      <c r="C39" s="24">
-        <f>(NPV($B39,$C$27:$G$27)+($G$27*(1+C$38)/($B39-C$38))/(1+$B39)^5-NetDebt)/Shares</f>
-        <v>47.39403874756321</v>
-      </c>
-      <c r="D39" s="24">
-        <f>(NPV($B39,$C$27:$G$27)+($G$27*(1+D$38)/($B39-D$38))/(1+$B39)^5-NetDebt)/Shares</f>
-        <v>50.53195287280684</v>
-      </c>
-      <c r="E39" s="24">
-        <f>(NPV($B39,$C$27:$G$27)+($G$27*(1+E$38)/($B39-E$38))/(1+$B39)^5-NetDebt)/Shares</f>
-        <v>54.253014020024786</v>
-      </c>
-      <c r="F39" s="24">
-        <f>(NPV($B39,$C$27:$G$27)+($G$27*(1+F$38)/($B39-F$38))/(1+$B39)^5-NetDebt)/Shares</f>
-        <v>58.73643147685507</v>
-      </c>
-      <c r="G39" s="24">
-        <f>(NPV($B39,$C$27:$G$27)+($G$27*(1+G$38)/($B39-G$38))/(1+$B39)^5-NetDebt)/Shares</f>
-        <v>64.24322657733528</v>
+      <c r="C39" s="9">
+        <f>(NPV($B39,$C$27:$G$27)*(1+$B39)^0.5+($G$27*(1+C$38)/($B39-C$38))/(1+$B39)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>45.5914522961236</v>
+      </c>
+      <c r="D39" s="9">
+        <f>(NPV($B39,$C$27:$G$27)*(1+$B39)^0.5+($G$27*(1+D$38)/($B39-D$38))/(1+$B39)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>48.689571144366184</v>
+      </c>
+      <c r="E39" s="9">
+        <f>(NPV($B39,$C$27:$G$27)*(1+$B39)^0.5+($G$27*(1+E$38)/($B39-E$38))/(1+$B39)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>52.363441497578606</v>
+      </c>
+      <c r="F39" s="9">
+        <f>(NPV($B39,$C$27:$G$27)*(1+$B39)^0.5+($G$27*(1+F$38)/($B39-F$38))/(1+$B39)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>56.78999989693163</v>
+      </c>
+      <c r="G39" s="9">
+        <f>(NPV($B39,$C$27:$G$27)*(1+$B39)^0.5+($G$27*(1+G$38)/($B39-G$38))/(1+$B39)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>62.22695738310345</v>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="30">
+      <c r="B40" s="22">
         <f>WACC+-0.005</f>
         <v>0.08881</v>
       </c>
-      <c r="C40" s="24">
-        <f>(NPV($B40,$C$27:$G$27)+($G$27*(1+C$38)/($B40-C$38))/(1+$B40)^5-NetDebt)/Shares</f>
-        <v>43.98434802278164</v>
-      </c>
-      <c r="D40" s="24">
-        <f>(NPV($B40,$C$27:$G$27)+($G$27*(1+D$38)/($B40-D$38))/(1+$B40)^5-NetDebt)/Shares</f>
-        <v>46.61731181734158</v>
-      </c>
-      <c r="E40" s="24">
-        <f>(NPV($B40,$C$27:$G$27)+($G$27*(1+E$38)/($B40-E$38))/(1+$B40)^5-NetDebt)/Shares</f>
-        <v>49.69798242954478</v>
-      </c>
-      <c r="F40" s="24">
-        <f>(NPV($B40,$C$27:$G$27)+($G$27*(1+F$38)/($B40-F$38))/(1+$B40)^5-NetDebt)/Shares</f>
-        <v>53.35116198287474</v>
-      </c>
-      <c r="G40" s="24">
-        <f>(NPV($B40,$C$27:$G$27)+($G$27*(1+G$38)/($B40-G$38))/(1+$B40)^5-NetDebt)/Shares</f>
-        <v>57.75279053299431</v>
+      <c r="C40" s="9">
+        <f>(NPV($B40,$C$27:$G$27)*(1+$B40)^0.5+($G$27*(1+C$38)/($B40-C$38))/(1+$B40)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>42.33016460969446</v>
+      </c>
+      <c r="D40" s="9">
+        <f>(NPV($B40,$C$27:$G$27)*(1+$B40)^0.5+($G$27*(1+D$38)/($B40-D$38))/(1+$B40)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>44.93572642232576</v>
+      </c>
+      <c r="E40" s="9">
+        <f>(NPV($B40,$C$27:$G$27)*(1+$B40)^0.5+($G$27*(1+E$38)/($B40-E$38))/(1+$B40)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>47.98433564400847</v>
+      </c>
+      <c r="F40" s="9">
+        <f>(NPV($B40,$C$27:$G$27)*(1+$B40)^0.5+($G$27*(1+F$38)/($B40-F$38))/(1+$B40)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>51.599495548033225</v>
+      </c>
+      <c r="G40" s="9">
+        <f>(NPV($B40,$C$27:$G$27)*(1+$B40)^0.5+($G$27*(1+G$38)/($B40-G$38))/(1+$B40)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>55.95531513327595</v>
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="30">
+      <c r="B41" s="22">
         <f>WACC+0</f>
         <v>0.09381</v>
       </c>
-      <c r="C41" s="24">
-        <f>(NPV($B41,$C$27:$G$27)+($G$27*(1+C$38)/($B41-C$38))/(1+$B41)^5-NetDebt)/Shares</f>
-        <v>41.03769707161954</v>
-      </c>
-      <c r="D41" s="24">
-        <f>(NPV($B41,$C$27:$G$27)+($G$27*(1+D$38)/($B41-D$38))/(1+$B41)^5-NetDebt)/Shares</f>
-        <v>43.27260312635998</v>
-      </c>
-      <c r="E41" s="24">
-        <f>(NPV($B41,$C$27:$G$27)+($G$27*(1+E$38)/($B41-E$38))/(1+$B41)^5-NetDebt)/Shares</f>
-        <v>45.85775303860559</v>
-      </c>
-      <c r="F41" s="24">
-        <f>(NPV($B41,$C$27:$G$27)+($G$27*(1+F$38)/($B41-F$38))/(1+$B41)^5-NetDebt)/Shares</f>
-        <v>48.882479538548104</v>
-      </c>
-      <c r="G41" s="24">
-        <f>(NPV($B41,$C$27:$G$27)+($G$27*(1+G$38)/($B41-G$38))/(1+$B41)^5-NetDebt)/Shares</f>
-        <v>52.469318378193755</v>
+      <c r="C41" s="9">
+        <f>(NPV($B41,$C$27:$G$27)*(1+$B41)^0.5+($G$27*(1+C$38)/($B41-C$38))/(1+$B41)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>39.51230863644887</v>
+      </c>
+      <c r="D41" s="9">
+        <f>(NPV($B41,$C$27:$G$27)*(1+$B41)^0.5+($G$27*(1+D$38)/($B41-D$38))/(1+$B41)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>41.72902771796434</v>
+      </c>
+      <c r="E41" s="9">
+        <f>(NPV($B41,$C$27:$G$27)*(1+$B41)^0.5+($G$27*(1+E$38)/($B41-E$38))/(1+$B41)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>44.293140480958506</v>
+      </c>
+      <c r="F41" s="9">
+        <f>(NPV($B41,$C$27:$G$27)*(1+$B41)^0.5+($G$27*(1+F$38)/($B41-F$38))/(1+$B41)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>47.29325269353507</v>
+      </c>
+      <c r="G41" s="9">
+        <f>(NPV($B41,$C$27:$G$27)*(1+$B41)^0.5+($G$27*(1+G$38)/($B41-G$38))/(1+$B41)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>50.85090294970513</v>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="30">
+      <c r="B42" s="22">
         <f>WACC+0.005</f>
         <v>0.09881000000000001</v>
       </c>
-      <c r="C42" s="24">
-        <f>(NPV($B42,$C$27:$G$27)+($G$27*(1+C$38)/($B42-C$38))/(1+$B42)^5-NetDebt)/Shares</f>
-        <v>38.465933352713236</v>
-      </c>
-      <c r="D42" s="24">
-        <f>(NPV($B42,$C$27:$G$27)+($G$27*(1+D$38)/($B42-D$38))/(1+$B42)^5-NetDebt)/Shares</f>
-        <v>40.381982514036416</v>
-      </c>
-      <c r="E42" s="24">
-        <f>(NPV($B42,$C$27:$G$27)+($G$27*(1+E$38)/($B42-E$38))/(1+$B42)^5-NetDebt)/Shares</f>
-        <v>42.576486719876854</v>
-      </c>
-      <c r="F42" s="24">
-        <f>(NPV($B42,$C$27:$G$27)+($G$27*(1+F$38)/($B42-F$38))/(1+$B42)^5-NetDebt)/Shares</f>
-        <v>45.114903197436526</v>
-      </c>
-      <c r="G42" s="24">
-        <f>(NPV($B42,$C$27:$G$27)+($G$27*(1+G$38)/($B42-G$38))/(1+$B42)^5-NetDebt)/Shares</f>
-        <v>48.08494975109885</v>
+      <c r="C42" s="9">
+        <f>(NPV($B42,$C$27:$G$27)*(1+$B42)^0.5+($G$27*(1+C$38)/($B42-C$38))/(1+$B42)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>37.05345225173073</v>
+      </c>
+      <c r="D42" s="9">
+        <f>(NPV($B42,$C$27:$G$27)*(1+$B42)^0.5+($G$27*(1+D$38)/($B42-D$38))/(1+$B42)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>38.958247909174</v>
+      </c>
+      <c r="E42" s="9">
+        <f>(NPV($B42,$C$27:$G$27)*(1+$B42)^0.5+($G$27*(1+E$38)/($B42-E$38))/(1+$B42)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>41.13986316514122</v>
+      </c>
+      <c r="F42" s="9">
+        <f>(NPV($B42,$C$27:$G$27)*(1+$B42)^0.5+($G$27*(1+F$38)/($B42-F$38))/(1+$B42)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>43.66337079784675</v>
+      </c>
+      <c r="G42" s="9">
+        <f>(NPV($B42,$C$27:$G$27)*(1+$B42)^0.5+($G$27*(1+G$38)/($B42-G$38))/(1+$B42)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>46.61597341995979</v>
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="30">
+      <c r="B43" s="22">
         <f>WACC+0.01</f>
         <v>0.10381</v>
       </c>
-      <c r="C43" s="24">
-        <f>(NPV($B43,$C$27:$G$27)+($G$27*(1+C$38)/($B43-C$38))/(1+$B43)^5-NetDebt)/Shares</f>
-        <v>36.201941148015415</v>
-      </c>
-      <c r="D43" s="24">
-        <f>(NPV($B43,$C$27:$G$27)+($G$27*(1+D$38)/($B43-D$38))/(1+$B43)^5-NetDebt)/Shares</f>
-        <v>37.85900456016365</v>
-      </c>
-      <c r="E43" s="24">
-        <f>(NPV($B43,$C$27:$G$27)+($G$27*(1+E$38)/($B43-E$38))/(1+$B43)^5-NetDebt)/Shares</f>
-        <v>39.74057188941638</v>
-      </c>
-      <c r="F43" s="24">
-        <f>(NPV($B43,$C$27:$G$27)+($G$27*(1+F$38)/($B43-F$38))/(1+$B43)^5-NetDebt)/Shares</f>
-        <v>41.895583097357196</v>
-      </c>
-      <c r="G43" s="24">
-        <f>(NPV($B43,$C$27:$G$27)+($G$27*(1+G$38)/($B43-G$38))/(1+$B43)^5-NetDebt)/Shares</f>
-        <v>44.38831742204161</v>
+      <c r="C43" s="9">
+        <f>(NPV($B43,$C$27:$G$27)*(1+$B43)^0.5+($G$27*(1+C$38)/($B43-C$38))/(1+$B43)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>34.8893126276283</v>
+      </c>
+      <c r="D43" s="9">
+        <f>(NPV($B43,$C$27:$G$27)*(1+$B43)^0.5+($G$27*(1+D$38)/($B43-D$38))/(1+$B43)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>36.54038736788702</v>
+      </c>
+      <c r="E43" s="9">
+        <f>(NPV($B43,$C$27:$G$27)*(1+$B43)^0.5+($G$27*(1+E$38)/($B43-E$38))/(1+$B43)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>38.41515466203531</v>
+      </c>
+      <c r="F43" s="9">
+        <f>(NPV($B43,$C$27:$G$27)*(1+$B43)^0.5+($G$27*(1+F$38)/($B43-F$38))/(1+$B43)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>40.56237760131486</v>
+      </c>
+      <c r="G43" s="9">
+        <f>(NPV($B43,$C$27:$G$27)*(1+$B43)^0.5+($G$27*(1+G$38)/($B43-G$38))/(1+$B43)^4.5-NetDebt-Minorities+Associates)/Shares</f>
+        <v>43.04610311688018</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="I3:K3"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="I19:K19"/>
     <mergeCell ref="B22:H22"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B37:H37"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="I19:K19"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="I26:K26"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="C39:G43">
     <cfRule type="colorScale" priority="1">
@@ -3424,7 +3694,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3439,33 +3709,33 @@
         <v>64</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>61</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" t="s">
         <v>65</v>
       </c>
-      <c r="C4" s="23">
+      <c r="C4" s="7">
         <f>RevGrowthMy</f>
         <v>0.16</v>
       </c>
-      <c r="D4" s="23">
+      <c r="D4" s="7">
         <f>EbitdaMarginMy</f>
         <v>0.26</v>
       </c>
@@ -3481,20 +3751,20 @@
         <f>(PeerEVEBITDA*F4-NetDebt)/Shares</f>
         <v>40.708</v>
       </c>
-      <c r="H4" s="23">
+      <c r="H4" s="7">
         <f>G4/Price-1</f>
         <v>-0.09537777777777778</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="s">
-        <v>157</v>
-      </c>
-      <c r="C5" s="23">
+        <v>170</v>
+      </c>
+      <c r="C5" s="7">
         <f>RevGrowthMy*1.25</f>
         <v>0.2</v>
       </c>
-      <c r="D5" s="23">
+      <c r="D5" s="7">
         <f>EbitdaMarginMy+0.03</f>
         <v>0.29000000000000004</v>
       </c>
@@ -3510,20 +3780,20 @@
         <f>(PeerEVEBITDA*F5-NetDebt)/Shares</f>
         <v>46.74000000000001</v>
       </c>
-      <c r="H5" s="23">
+      <c r="H5" s="7">
         <f>G5/Price-1</f>
         <v>0.03866666666666685</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="s">
-        <v>158</v>
-      </c>
-      <c r="C6" s="23">
+        <v>171</v>
+      </c>
+      <c r="C6" s="7">
         <f>RevGrowthMy*0.7</f>
         <v>0.11199999999999999</v>
       </c>
-      <c r="D6" s="23">
+      <c r="D6" s="7">
         <f>EbitdaMarginMy-0.04</f>
         <v>0.22</v>
       </c>
@@ -3539,39 +3809,39 @@
         <f>(PeerEVEBITDA*F6-NetDebt)/Shares</f>
         <v>33.303200000000004</v>
       </c>
-      <c r="H6" s="23">
+      <c r="H6" s="7">
         <f>G6/Price-1</f>
         <v>-0.25992888888888876</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
+      <c r="B8" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
     </row>
     <row r="9">
-      <c r="B9" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>162</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>163</v>
+      <c r="B9" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
       <c r="C10" s="5">
         <f>(PeerEVEBITDA*(PriorRev*(1+RevGrowthMy*0.8)*EbitdaMarginMy)-NetDebt)/Shares</f>
@@ -3622,7 +3892,7 @@
     </row>
     <row r="13">
       <c r="B13" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="C13" s="5">
         <f>(PeerEVEBITDA*(PriorRev*(1+RevGrowthMy)*EbitdaMarginMy)-NetDebt*1.2)/Shares</f>
@@ -3639,7 +3909,7 @@
     </row>
     <row r="14">
       <c r="B14" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
       <c r="C14" s="5">
         <f>(PeerEVEBITDA*(PriorRev*(1+RevGrowthMy)*EbitdaMarginMy)-NetDebt)/Shares*1.2</f>
@@ -3681,7 +3951,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3741,10 +4011,10 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10">
@@ -3752,7 +4022,7 @@
         <f>INDEX(KpiNames,1,MATCH(SelectedSector,SectorList,0))</f>
         <v>ARR ($M)</v>
       </c>
-      <c r="B10" s="22">
+      <c r="B10" s="3">
         <f>INDEX(KpiValues,1,MATCH(SelectedSector,SectorList,0))</f>
         <v>1200</v>
       </c>
@@ -3762,7 +4032,7 @@
         <f>INDEX(KpiNames,2,MATCH(SelectedSector,SectorList,0))</f>
         <v>Net Rev Retention (%)</v>
       </c>
-      <c r="B11" s="22">
+      <c r="B11" s="3">
         <f>INDEX(KpiValues,2,MATCH(SelectedSector,SectorList,0))</f>
         <v>118</v>
       </c>
@@ -3772,7 +4042,7 @@
         <f>INDEX(KpiNames,3,MATCH(SelectedSector,SectorList,0))</f>
         <v>Rule of 40 (%)</v>
       </c>
-      <c r="B12" s="22">
+      <c r="B12" s="3">
         <f>INDEX(KpiValues,3,MATCH(SelectedSector,SectorList,0))</f>
         <v>46</v>
       </c>
@@ -3782,7 +4052,7 @@
         <f>INDEX(KpiNames,4,MATCH(SelectedSector,SectorList,0))</f>
         <v>Gross Margin (%)</v>
       </c>
-      <c r="B13" s="22">
+      <c r="B13" s="3">
         <f>INDEX(KpiValues,4,MATCH(SelectedSector,SectorList,0))</f>
         <v>78</v>
       </c>
@@ -3792,22 +4062,22 @@
         <f>INDEX(KpiNames,5,MATCH(SelectedSector,SectorList,0))</f>
         <v>CAC Payback (mo)</v>
       </c>
-      <c r="B14" s="22">
+      <c r="B14" s="3">
         <f>INDEX(KpiValues,5,MATCH(SelectedSector,SectorList,0))</f>
         <v>14</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="B18" s="1">
         <f>ConsNI</f>
@@ -3816,7 +4086,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="B19" s="1">
         <f>(RevMy-ConsRev)*NiMarginMy</f>
@@ -3825,7 +4095,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="B20" s="1">
         <f>NiMy-ConsNI-((RevMy-ConsRev)*NiMarginMy)</f>
@@ -3834,7 +4104,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="B21" s="1">
         <f>NiMy</f>
@@ -3859,7 +4129,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3871,294 +4141,294 @@
       <c r="I1" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="s">
-        <v>175</v>
-      </c>
-      <c r="C3" s="21" t="s">
+      <c r="A3" s="28" t="s">
+        <v>188</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="D3" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E3" s="21" t="s">
-        <v>176</v>
-      </c>
-      <c r="F3" s="21" t="s">
-        <v>177</v>
-      </c>
-      <c r="G3" s="21" t="s">
-        <v>178</v>
-      </c>
-      <c r="H3" s="21" t="s">
+      <c r="E3" s="10" t="s">
+        <v>189</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="H3" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="I3" s="21" t="s">
-        <v>179</v>
+      <c r="I3" s="10" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20"/>
+      <c r="A4" s="28"/>
       <c r="C4" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="D4" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="E4" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="F4" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="G4" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="H4" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="I4" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20"/>
+      <c r="A5" s="28"/>
       <c r="C5" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="D5" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="E5" t="s">
+        <v>202</v>
+      </c>
+      <c r="F5" t="s">
+        <v>203</v>
+      </c>
+      <c r="G5" t="s">
+        <v>204</v>
+      </c>
+      <c r="H5" t="s">
+        <v>205</v>
+      </c>
+      <c r="I5" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="28"/>
+      <c r="C6" t="s">
+        <v>206</v>
+      </c>
+      <c r="D6" t="s">
+        <v>207</v>
+      </c>
+      <c r="E6" t="s">
+        <v>208</v>
+      </c>
+      <c r="F6" t="s">
+        <v>209</v>
+      </c>
+      <c r="G6" t="s">
+        <v>210</v>
+      </c>
+      <c r="H6" t="s">
+        <v>211</v>
+      </c>
+      <c r="I6" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="28"/>
+      <c r="C7" t="s">
+        <v>201</v>
+      </c>
+      <c r="D7" t="s">
+        <v>213</v>
+      </c>
+      <c r="E7" t="s">
+        <v>201</v>
+      </c>
+      <c r="F7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G7" t="s">
+        <v>214</v>
+      </c>
+      <c r="H7" t="s">
+        <v>215</v>
+      </c>
+      <c r="I7" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="28"/>
+      <c r="C8" t="s">
+        <v>217</v>
+      </c>
+      <c r="D8" t="s">
+        <v>218</v>
+      </c>
+      <c r="E8" t="s">
+        <v>219</v>
+      </c>
+      <c r="F8" t="s">
+        <v>220</v>
+      </c>
+      <c r="G8" t="s">
+        <v>221</v>
+      </c>
+      <c r="H8" t="s">
+        <v>222</v>
+      </c>
+      <c r="I8" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="28" t="s">
+        <v>223</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="E10" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F10" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G10" s="10" t="s">
         <v>191</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H10" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="I10" s="10" t="s">
         <v>192</v>
       </c>
-      <c r="I5" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="20"/>
-      <c r="C6" t="s">
-        <v>193</v>
-      </c>
-      <c r="D6" t="s">
-        <v>194</v>
-      </c>
-      <c r="E6" t="s">
-        <v>195</v>
-      </c>
-      <c r="F6" t="s">
-        <v>196</v>
-      </c>
-      <c r="G6" t="s">
-        <v>197</v>
-      </c>
-      <c r="H6" t="s">
-        <v>198</v>
-      </c>
-      <c r="I6" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="20"/>
-      <c r="C7" t="s">
-        <v>188</v>
-      </c>
-      <c r="D7" t="s">
-        <v>200</v>
-      </c>
-      <c r="E7" t="s">
-        <v>188</v>
-      </c>
-      <c r="F7" t="s">
-        <v>199</v>
-      </c>
-      <c r="G7" t="s">
-        <v>201</v>
-      </c>
-      <c r="H7" t="s">
-        <v>202</v>
-      </c>
-      <c r="I7" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="20"/>
-      <c r="C8" t="s">
-        <v>204</v>
-      </c>
-      <c r="D8" t="s">
-        <v>205</v>
-      </c>
-      <c r="E8" t="s">
-        <v>206</v>
-      </c>
-      <c r="F8" t="s">
-        <v>207</v>
-      </c>
-      <c r="G8" t="s">
-        <v>208</v>
-      </c>
-      <c r="H8" t="s">
-        <v>209</v>
-      </c>
-      <c r="I8" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="20" t="s">
-        <v>210</v>
-      </c>
-      <c r="C10" s="21" t="s">
-        <v>3</v>
-      </c>
-      <c r="D10" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="E10" s="21" t="s">
-        <v>176</v>
-      </c>
-      <c r="F10" s="21" t="s">
-        <v>177</v>
-      </c>
-      <c r="G10" s="21" t="s">
-        <v>178</v>
-      </c>
-      <c r="H10" s="21" t="s">
+    </row>
+    <row r="11">
+      <c r="A11" s="28"/>
+      <c r="C11" s="36">
+        <v>1200</v>
+      </c>
+      <c r="D11" s="36">
+        <v>4.5</v>
+      </c>
+      <c r="E11" s="36">
+        <v>22</v>
+      </c>
+      <c r="F11" s="36">
+        <v>1.08</v>
+      </c>
+      <c r="G11" s="36">
+        <v>3.2</v>
+      </c>
+      <c r="H11" s="36">
+        <v>520</v>
+      </c>
+      <c r="I11" s="36">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="28"/>
+      <c r="C12" s="36">
+        <v>118</v>
+      </c>
+      <c r="D12" s="36">
+        <v>42</v>
+      </c>
+      <c r="E12" s="36">
+        <v>12</v>
+      </c>
+      <c r="F12" s="36">
+        <v>84</v>
+      </c>
+      <c r="G12" s="36">
+        <v>58</v>
+      </c>
+      <c r="H12" s="36">
+        <v>68</v>
+      </c>
+      <c r="I12" s="36">
         <v>55</v>
       </c>
-      <c r="I10" s="21" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="20"/>
-      <c r="C11" s="19">
-        <v>1200</v>
-      </c>
-      <c r="D11" s="19">
-        <v>4.5</v>
-      </c>
-      <c r="E11" s="19">
-        <v>22</v>
-      </c>
-      <c r="F11" s="19">
-        <v>1.08</v>
-      </c>
-      <c r="G11" s="19">
-        <v>3.2</v>
-      </c>
-      <c r="H11" s="19">
-        <v>520</v>
-      </c>
-      <c r="I11" s="19">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="20"/>
-      <c r="C12" s="19">
-        <v>118</v>
-      </c>
-      <c r="D12" s="19">
-        <v>42</v>
-      </c>
-      <c r="E12" s="19">
-        <v>12</v>
-      </c>
-      <c r="F12" s="19">
-        <v>84</v>
-      </c>
-      <c r="G12" s="19">
-        <v>58</v>
-      </c>
-      <c r="H12" s="19">
-        <v>68</v>
-      </c>
-      <c r="I12" s="19">
-        <v>55</v>
-      </c>
     </row>
     <row r="13">
-      <c r="A13" s="20"/>
-      <c r="C13" s="19">
+      <c r="A13" s="28"/>
+      <c r="C13" s="36">
         <v>46</v>
       </c>
-      <c r="D13" s="19">
+      <c r="D13" s="36">
         <v>5.2</v>
       </c>
-      <c r="E13" s="19">
+      <c r="E13" s="36">
         <v>340</v>
       </c>
-      <c r="F13" s="19">
+      <c r="F13" s="36">
         <v>2300</v>
       </c>
-      <c r="G13" s="19">
+      <c r="G13" s="36">
         <v>13.5</v>
       </c>
-      <c r="H13" s="19">
+      <c r="H13" s="36">
         <v>12.5</v>
       </c>
-      <c r="I13" s="19">
+      <c r="I13" s="36">
         <v>20</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="20"/>
-      <c r="C14" s="19">
+      <c r="A14" s="28"/>
+      <c r="C14" s="36">
         <v>78</v>
       </c>
-      <c r="D14" s="19">
+      <c r="D14" s="36">
         <v>1450</v>
       </c>
-      <c r="E14" s="19">
+      <c r="E14" s="36">
         <v>74</v>
       </c>
-      <c r="F14" s="19">
+      <c r="F14" s="36">
         <v>16</v>
       </c>
-      <c r="G14" s="19">
+      <c r="G14" s="36">
         <v>12.2</v>
       </c>
-      <c r="H14" s="19">
+      <c r="H14" s="36">
         <v>9.4</v>
       </c>
-      <c r="I14" s="19">
+      <c r="I14" s="36">
         <v>18</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="20"/>
-      <c r="C15" s="19">
+      <c r="A15" s="28"/>
+      <c r="C15" s="36">
         <v>14</v>
       </c>
-      <c r="D15" s="19">
+      <c r="D15" s="36">
         <v>31</v>
       </c>
-      <c r="E15" s="19">
+      <c r="E15" s="36">
         <v>28</v>
       </c>
-      <c r="F15" s="19">
+      <c r="F15" s="36">
         <v>13</v>
       </c>
-      <c r="G15" s="19">
+      <c r="G15" s="36">
         <v>7</v>
       </c>
-      <c r="H15" s="19">
+      <c r="H15" s="36">
         <v>11</v>
       </c>
-      <c r="I15" s="19">
+      <c r="I15" s="36">
         <v>14</v>
       </c>
     </row>
@@ -4167,4 +4437,294 @@
     <mergeCell ref="A1:I1"/>
   </mergeCells>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H22"/>
+  <sheetFormatPr defaultColWidth="8.42578125" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="26.42578125" customWidth="1"/>
+    <col min="3" max="8" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="42" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="42" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="42" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="42" t="s">
+        <v>225</v>
+      </c>
+      <c r="E3" s="42" t="s">
+        <v>226</v>
+      </c>
+      <c r="F3" s="42" t="s">
+        <v>227</v>
+      </c>
+      <c r="G3" s="42" t="s">
+        <v>228</v>
+      </c>
+      <c r="H3" s="42" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>230</v>
+      </c>
+      <c r="C4" s="5"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="33"/>
+      <c r="G4" s="33"/>
+      <c r="H4" s="33"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>231</v>
+      </c>
+      <c r="C5" s="5"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="33"/>
+      <c r="G5" s="33"/>
+      <c r="H5" s="33"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>232</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>233</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="33"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="33"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>234</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>235</v>
+      </c>
+      <c r="C9" s="5"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="33"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="33"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>236</v>
+      </c>
+      <c r="C10" s="5"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="33"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="33"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>237</v>
+      </c>
+      <c r="C11" s="5"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="33"/>
+      <c r="G11" s="33"/>
+      <c r="H11" s="33"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="44" t="str">
+        <f>IFERROR(MEDIAN(F4:F11),"")</f>
+        <v/>
+      </c>
+      <c r="G13" s="44" t="str">
+        <f>IFERROR(MEDIAN(G4:G11),"")</f>
+        <v/>
+      </c>
+      <c r="H13" s="44" t="str">
+        <f>IFERROR(MEDIAN(H4:H11),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>244</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="11" t="str">
+        <f>G13</f>
+        <v/>
+      </c>
+      <c r="C17" s="1">
+        <f>ConsEBITDA</f>
+        <v>295</v>
+      </c>
+      <c r="D17" s="1" t="str">
+        <f>IFERROR(G13*ConsEBITDA,"")</f>
+        <v/>
+      </c>
+      <c r="E17" s="5" t="str">
+        <f>IFERROR((D17-NetDebt-Minorities+Associates)/Shares,"")</f>
+        <v/>
+      </c>
+      <c r="F17" s="7" t="str">
+        <f>IFERROR(E17/Price-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>245</v>
+      </c>
+      <c r="B18" s="11" t="str">
+        <f>F13</f>
+        <v/>
+      </c>
+      <c r="C18" s="1">
+        <f>ConsRev</f>
+        <v>1150</v>
+      </c>
+      <c r="D18" s="1" t="str">
+        <f>IFERROR(F13*ConsRev,"")</f>
+        <v/>
+      </c>
+      <c r="E18" s="5" t="str">
+        <f>IFERROR((D18-NetDebt-Minorities+Associates)/Shares,"")</f>
+        <v/>
+      </c>
+      <c r="F18" s="7" t="str">
+        <f>IFERROR(E18/Price-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="11" t="str">
+        <f>H13</f>
+        <v/>
+      </c>
+      <c r="C19" s="1">
+        <f>ConsNI</f>
+        <v>150</v>
+      </c>
+      <c r="D19" s="1" t="str">
+        <f>IFERROR(H13*ConsNI,"")</f>
+        <v/>
+      </c>
+      <c r="E19" s="5" t="str">
+        <f>IFERROR(D19/Shares,"")</f>
+        <v/>
+      </c>
+      <c r="F19" s="7" t="str">
+        <f>IFERROR(E19/Price-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="47" t="s">
+        <v>246</v>
+      </c>
+      <c r="B20" s="45"/>
+      <c r="C20" s="43"/>
+      <c r="D20" s="43"/>
+      <c r="E20" s="38" t="str">
+        <f>IFERROR(AVERAGE(E17:E19),"")</f>
+        <v/>
+      </c>
+      <c r="F20" s="46" t="str">
+        <f>IFERROR(E20/Price-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="19" t="s">
+        <v>247</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
+</worksheet>
 </file>
</xml_diff>